<commit_message>
minor Updates to ReadMe
</commit_message>
<xml_diff>
--- a/__ReadMe.xlsx
+++ b/__ReadMe.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10414"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10512"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://alleninstitute.sharepoint.com/sites/MammalianM1/Shared Documents/General/Species/Evo-M1-Trait-Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="53" documentId="6_{3E294B1E-BE69-A04D-8F66-E6809E46817C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{47D15A47-F99B-7246-8B5B-2AFC1BCCAE91}"/>
+  <xr:revisionPtr revIDLastSave="55" documentId="6_{3E294B1E-BE69-A04D-8F66-E6809E46817C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1936AC6B-01E4-6049-903E-6E6C4FEF2BF5}"/>
   <bookViews>
-    <workbookView xWindow="35000" yWindow="-5960" windowWidth="49660" windowHeight="24360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34560" yWindow="-7080" windowWidth="38400" windowHeight="19680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Pipeline" sheetId="3" r:id="rId2"/>
-    <sheet name="Conflcts" sheetId="4" r:id="rId3"/>
+    <sheet name="Conflicts" sheetId="4" r:id="rId3"/>
     <sheet name="FileList" sheetId="6" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -1695,7 +1695,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:37" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:37" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>38</v>
       </c>
@@ -5025,7 +5025,7 @@
         <v>2014</v>
       </c>
       <c r="H44" t="str">
-        <f>_xlfn.TEXTAFTER(A44,"https://doi.org/")</f>
+        <f t="shared" ref="H44:H49" si="51">_xlfn.TEXTAFTER(A44,"https://doi.org/")</f>
         <v>10.1371/journal.pbio.1002000</v>
       </c>
       <c r="J44" s="1" t="s">
@@ -5068,11 +5068,11 @@
         <v>0</v>
       </c>
       <c r="C45" s="2" t="str">
-        <f t="shared" ref="C45" si="51">D45 &amp; IF(E45&lt;&gt;"", "_" &amp; E45, "_") &amp; IF(F45&lt;&gt;"", "_" &amp; F45, "_") &amp; IF(G45&lt;&gt;"", "_" &amp; G45, "")</f>
+        <f t="shared" ref="C45" si="52">D45 &amp; IF(E45&lt;&gt;"", "_" &amp; E45, "_") &amp; IF(F45&lt;&gt;"", "_" &amp; F45, "_") &amp; IF(G45&lt;&gt;"", "_" &amp; G45, "")</f>
         <v>Lewitus_etal_2014</v>
       </c>
       <c r="D45" s="2" t="str">
-        <f t="shared" ref="D45" si="52">SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTBEFORE(A45,","), "-", ""), " ", "")</f>
+        <f t="shared" ref="D45" si="53">SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTBEFORE(A45,","), "-", ""), " ", "")</f>
         <v>Lewitus</v>
       </c>
       <c r="E45" s="2" t="str">
@@ -5080,22 +5080,22 @@
         <v>etal</v>
       </c>
       <c r="F45" s="2" t="str">
-        <f t="shared" ref="F45" si="53">_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(A45, "("), ")")</f>
+        <f t="shared" ref="F45" si="54">_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(A45, "("), ")")</f>
         <v>2014</v>
       </c>
       <c r="H45" t="str">
-        <f>_xlfn.TEXTAFTER(A45,"https://doi.org/")</f>
+        <f t="shared" si="51"/>
         <v>10.1371/journal.pbio.1002000</v>
       </c>
       <c r="J45" s="1" t="s">
         <v>224</v>
       </c>
       <c r="K45" s="1" t="str">
-        <f t="shared" ref="K45" si="54">TRIM(_xlfn.TEXTJOIN("_",FALSE,C45,(SUBSTITUTE(SUBSTITUTE(J45," ",""), "_", ""))))</f>
+        <f t="shared" ref="K45" si="55">TRIM(_xlfn.TEXTJOIN("_",FALSE,C45,(SUBSTITUTE(SUBSTITUTE(J45," ",""), "_", ""))))</f>
         <v>Lewitus_etal_2014_TableS8</v>
       </c>
       <c r="L45" s="1" t="str">
-        <f t="shared" ref="L45" si="55">IF(ISBLANK(I45),TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTJOIN("_", FALSE, H45, SUBSTITUTE(J45,"_", "")), "/", "%2F"), ":", "%3A"), " ", "")),TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTJOIN("_", FALSE, I45, SUBSTITUTE(J45,"_", "")), "/", "%2F"), ":", "%3A"), " ", "")))</f>
+        <f t="shared" ref="L45" si="56">IF(ISBLANK(I45),TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTJOIN("_", FALSE, H45, SUBSTITUTE(J45,"_", "")), "/", "%2F"), ":", "%3A"), " ", "")),TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTJOIN("_", FALSE, I45, SUBSTITUTE(J45,"_", "")), "/", "%2F"), ":", "%3A"), " ", "")))</f>
         <v>10.1371%2Fjournal.pbio.1002000_TableS8</v>
       </c>
       <c r="O45" t="str">
@@ -5127,11 +5127,11 @@
         <v>4</v>
       </c>
       <c r="C46" s="7" t="str">
-        <f t="shared" ref="C46" si="56">D46 &amp; IF(E46&lt;&gt;"", "_" &amp; E46, "_") &amp; IF(F46&lt;&gt;"", "_" &amp; F46, "_") &amp; IF(G46&lt;&gt;"", "_" &amp; G46, "")</f>
+        <f t="shared" ref="C46" si="57">D46 &amp; IF(E46&lt;&gt;"", "_" &amp; E46, "_") &amp; IF(F46&lt;&gt;"", "_" &amp; F46, "_") &amp; IF(G46&lt;&gt;"", "_" &amp; G46, "")</f>
         <v>Lewitus_etal_2013</v>
       </c>
       <c r="D46" s="7" t="str">
-        <f t="shared" ref="D46" si="57">SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTBEFORE(A46,","), "-", ""), " ", "")</f>
+        <f t="shared" ref="D46" si="58">SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTBEFORE(A46,","), "-", ""), " ", "")</f>
         <v>Lewitus</v>
       </c>
       <c r="E46" s="2" t="str">
@@ -5142,19 +5142,19 @@
         <v>etal</v>
       </c>
       <c r="F46" s="7" t="str">
-        <f t="shared" ref="F46" si="58">_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(A46, "("), ")")</f>
+        <f t="shared" ref="F46" si="59">_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(A46, "("), ")")</f>
         <v>2013</v>
       </c>
       <c r="G46" s="7"/>
       <c r="H46" s="6" t="str">
-        <f>_xlfn.TEXTAFTER(A46,"https://doi.org/")</f>
+        <f t="shared" si="51"/>
         <v>10.3389/fnhum.2013.00424</v>
       </c>
       <c r="J46" s="6" t="s">
         <v>227</v>
       </c>
       <c r="K46" s="6" t="str">
-        <f t="shared" ref="K46" si="59">TRIM(_xlfn.TEXTJOIN("_",FALSE,C46,(SUBSTITUTE(SUBSTITUTE(J46," ",""), "_", ""))))</f>
+        <f t="shared" ref="K46" si="60">TRIM(_xlfn.TEXTJOIN("_",FALSE,C46,(SUBSTITUTE(SUBSTITUTE(J46," ",""), "_", ""))))</f>
         <v>Lewitus_etal_2013_TableS2partial</v>
       </c>
       <c r="L46" s="8" t="str">
@@ -5187,11 +5187,11 @@
         <v>1</v>
       </c>
       <c r="C47" s="9" t="str">
-        <f t="shared" ref="C47" si="60">D47 &amp; IF(E47&lt;&gt;"", "_" &amp; E47, "_") &amp; IF(F47&lt;&gt;"", "_" &amp; F47, "_") &amp; IF(G47&lt;&gt;"", "_" &amp; G47, "")</f>
+        <f t="shared" ref="C47" si="61">D47 &amp; IF(E47&lt;&gt;"", "_" &amp; E47, "_") &amp; IF(F47&lt;&gt;"", "_" &amp; F47, "_") &amp; IF(G47&lt;&gt;"", "_" &amp; G47, "")</f>
         <v>Smaers_etal_2011</v>
       </c>
       <c r="D47" s="9" t="str">
-        <f t="shared" ref="D47" si="61">SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTBEFORE(A47,","), "-", ""), " ", "")</f>
+        <f t="shared" ref="D47" si="62">SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTBEFORE(A47,","), "-", ""), " ", "")</f>
         <v>Smaers</v>
       </c>
       <c r="E47" s="2" t="str">
@@ -5199,19 +5199,19 @@
         <v>etal</v>
       </c>
       <c r="F47" s="9" t="str">
-        <f t="shared" ref="F47" si="62">_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(A47, "("), ")")</f>
+        <f t="shared" ref="F47" si="63">_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(A47, "("), ")")</f>
         <v>2011</v>
       </c>
       <c r="G47" s="9"/>
       <c r="H47" t="str">
-        <f>_xlfn.TEXTAFTER(A47,"https://doi.org/")</f>
+        <f t="shared" si="51"/>
         <v>10.1159/000323671</v>
       </c>
       <c r="J47" s="5" t="s">
         <v>229</v>
       </c>
       <c r="K47" s="5" t="str">
-        <f t="shared" ref="K47" si="63">TRIM(_xlfn.TEXTJOIN("_",FALSE,C47,(SUBSTITUTE(SUBSTITUTE(J47," ",""), "_", ""))))</f>
+        <f t="shared" ref="K47" si="64">TRIM(_xlfn.TEXTJOIN("_",FALSE,C47,(SUBSTITUTE(SUBSTITUTE(J47," ",""), "_", ""))))</f>
         <v>Smaers_etal_2011_SupplementaryTable1</v>
       </c>
       <c r="L47" s="5" t="str">
@@ -5238,11 +5238,11 @@
         <v>1</v>
       </c>
       <c r="C48" s="9" t="str">
-        <f t="shared" ref="C48" si="64">D48 &amp; IF(E48&lt;&gt;"", "_" &amp; E48, "_") &amp; IF(F48&lt;&gt;"", "_" &amp; F48, "_") &amp; IF(G48&lt;&gt;"", "_" &amp; G48, "")</f>
+        <f t="shared" ref="C48" si="65">D48 &amp; IF(E48&lt;&gt;"", "_" &amp; E48, "_") &amp; IF(F48&lt;&gt;"", "_" &amp; F48, "_") &amp; IF(G48&lt;&gt;"", "_" &amp; G48, "")</f>
         <v>Smaers_etal_2011</v>
       </c>
       <c r="D48" s="9" t="str">
-        <f t="shared" ref="D48" si="65">SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTBEFORE(A48,","), "-", ""), " ", "")</f>
+        <f t="shared" ref="D48" si="66">SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTBEFORE(A48,","), "-", ""), " ", "")</f>
         <v>Smaers</v>
       </c>
       <c r="E48" s="2" t="str">
@@ -5250,19 +5250,19 @@
         <v>etal</v>
       </c>
       <c r="F48" s="9" t="str">
-        <f t="shared" ref="F48" si="66">_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(A48, "("), ")")</f>
+        <f t="shared" ref="F48" si="67">_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(A48, "("), ")")</f>
         <v>2011</v>
       </c>
       <c r="G48" s="9"/>
       <c r="H48" t="str">
-        <f>_xlfn.TEXTAFTER(A48,"https://doi.org/")</f>
+        <f t="shared" si="51"/>
         <v>10.1159/000323671</v>
       </c>
       <c r="J48" s="5" t="s">
         <v>231</v>
       </c>
       <c r="K48" s="5" t="str">
-        <f t="shared" ref="K48" si="67">TRIM(_xlfn.TEXTJOIN("_",FALSE,C48,(SUBSTITUTE(SUBSTITUTE(J48," ",""), "_", ""))))</f>
+        <f t="shared" ref="K48" si="68">TRIM(_xlfn.TEXTJOIN("_",FALSE,C48,(SUBSTITUTE(SUBSTITUTE(J48," ",""), "_", ""))))</f>
         <v>Smaers_etal_2011_SupplementaryTable2</v>
       </c>
       <c r="L48" s="5" t="str">
@@ -5289,27 +5289,27 @@
         <v>x</v>
       </c>
       <c r="C49" s="9" t="str">
-        <f t="shared" ref="C49:C53" si="68">D49 &amp; IF(E49&lt;&gt;"", "_" &amp; E49, "_") &amp; IF(F49&lt;&gt;"", "_" &amp; F49, "_") &amp; IF(G49&lt;&gt;"", "_" &amp; G49, "")</f>
+        <f t="shared" ref="C49:C53" si="69">D49 &amp; IF(E49&lt;&gt;"", "_" &amp; E49, "_") &amp; IF(F49&lt;&gt;"", "_" &amp; F49, "_") &amp; IF(G49&lt;&gt;"", "_" &amp; G49, "")</f>
         <v>Iwaniuk_etal_1999</v>
       </c>
       <c r="D49" s="9" t="str">
-        <f t="shared" ref="D49:D53" si="69">SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTBEFORE(A49,","), "-", ""), " ", "")</f>
+        <f t="shared" ref="D49:D53" si="70">SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTBEFORE(A49,","), "-", ""), " ", "")</f>
         <v>Iwaniuk</v>
       </c>
       <c r="E49" s="2" t="str">
-        <f t="shared" ref="E49:E53" si="70">IF(ISNUMBER(FIND("&amp;", A49)),
+        <f t="shared" ref="E49:E53" si="71">IF(ISNUMBER(FIND("&amp;", A49)),
     IF(LEN(A49)-LEN(SUBSTITUTE(A49, ",", ""))&gt;=6, "etal", MID(A49, SEARCH("&amp; ", A49)+2, SEARCH(",", A49, SEARCH("&amp; ", A49)+2) - SEARCH("&amp; ", A49)-2)),
     ""
 )</f>
         <v>etal</v>
       </c>
       <c r="F49" s="9" t="str">
-        <f t="shared" ref="F49:F52" si="71">_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(A49, "("), ")")</f>
+        <f t="shared" ref="F49:F52" si="72">_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(A49, "("), ")")</f>
         <v>1999</v>
       </c>
       <c r="G49" s="9"/>
       <c r="H49" t="str">
-        <f>_xlfn.TEXTAFTER(A49,"https://doi.org/")</f>
+        <f t="shared" si="51"/>
         <v>10.1016/s0166-4328(98)00151-x</v>
       </c>
       <c r="I49" s="5"/>
@@ -5317,7 +5317,7 @@
         <v>52</v>
       </c>
       <c r="K49" s="5" t="str">
-        <f t="shared" ref="K49:K52" si="72">TRIM(_xlfn.TEXTJOIN("_",FALSE,C49,(SUBSTITUTE(SUBSTITUTE(J49," ",""), "_", ""))))</f>
+        <f t="shared" ref="K49:K52" si="73">TRIM(_xlfn.TEXTJOIN("_",FALSE,C49,(SUBSTITUTE(SUBSTITUTE(J49," ",""), "_", ""))))</f>
         <v>Iwaniuk_etal_1999_Table1</v>
       </c>
       <c r="L49" s="5" t="str">
@@ -5350,27 +5350,27 @@
         <v>x</v>
       </c>
       <c r="C50" s="9" t="str">
-        <f t="shared" ref="C50" si="73">D50 &amp; IF(E50&lt;&gt;"", "_" &amp; E50, "_") &amp; IF(F50&lt;&gt;"", "_" &amp; F50, "_") &amp; IF(G50&lt;&gt;"", "_" &amp; G50, "")</f>
+        <f t="shared" ref="C50" si="74">D50 &amp; IF(E50&lt;&gt;"", "_" &amp; E50, "_") &amp; IF(F50&lt;&gt;"", "_" &amp; F50, "_") &amp; IF(G50&lt;&gt;"", "_" &amp; G50, "")</f>
         <v>Iwaniuk_etal_1999</v>
       </c>
       <c r="D50" s="9" t="str">
-        <f t="shared" ref="D50" si="74">SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTBEFORE(A50,","), "-", ""), " ", "")</f>
+        <f t="shared" ref="D50" si="75">SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTBEFORE(A50,","), "-", ""), " ", "")</f>
         <v>Iwaniuk</v>
       </c>
       <c r="E50" s="2" t="str">
-        <f t="shared" ref="E50" si="75">IF(ISNUMBER(FIND("&amp;", A50)),
+        <f t="shared" ref="E50" si="76">IF(ISNUMBER(FIND("&amp;", A50)),
     IF(LEN(A50)-LEN(SUBSTITUTE(A50, ",", ""))&gt;=6, "etal", MID(A50, SEARCH("&amp; ", A50)+2, SEARCH(",", A50, SEARCH("&amp; ", A50)+2) - SEARCH("&amp; ", A50)-2)),
     ""
 )</f>
         <v>etal</v>
       </c>
       <c r="F50" s="9" t="str">
-        <f t="shared" ref="F50" si="76">_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(A50, "("), ")")</f>
+        <f t="shared" ref="F50" si="77">_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(A50, "("), ")")</f>
         <v>1999</v>
       </c>
       <c r="G50" s="9"/>
       <c r="H50" t="str">
-        <f t="shared" ref="H50" si="77">_xlfn.TEXTAFTER(A50,"https://doi.org/")</f>
+        <f t="shared" ref="H50" si="78">_xlfn.TEXTAFTER(A50,"https://doi.org/")</f>
         <v>10.1016/s0166-4328(98)00151-x</v>
       </c>
       <c r="I50" s="5"/>
@@ -5378,7 +5378,7 @@
         <v>340</v>
       </c>
       <c r="K50" s="5" t="str">
-        <f t="shared" ref="K50" si="78">TRIM(_xlfn.TEXTJOIN("_",FALSE,C50,(SUBSTITUTE(SUBSTITUTE(J50," ",""), "_", ""))))</f>
+        <f t="shared" ref="K50" si="79">TRIM(_xlfn.TEXTJOIN("_",FALSE,C50,(SUBSTITUTE(SUBSTITUTE(J50," ",""), "_", ""))))</f>
         <v>Iwaniuk_etal_1999_References</v>
       </c>
       <c r="L50" s="5" t="str">
@@ -5411,19 +5411,19 @@
         <v>0</v>
       </c>
       <c r="C51" s="9" t="str">
-        <f t="shared" si="68"/>
+        <f t="shared" si="69"/>
         <v>Genoud_etal_2018</v>
       </c>
       <c r="D51" s="9" t="str">
-        <f t="shared" si="69"/>
+        <f t="shared" si="70"/>
         <v>Genoud</v>
       </c>
       <c r="E51" s="2" t="str">
-        <f t="shared" si="70"/>
+        <f t="shared" si="71"/>
         <v>etal</v>
       </c>
       <c r="F51" s="9" t="str">
-        <f t="shared" si="71"/>
+        <f t="shared" si="72"/>
         <v>2018</v>
       </c>
       <c r="G51" s="9"/>
@@ -5436,11 +5436,11 @@
         <v>220</v>
       </c>
       <c r="K51" s="5" t="str">
-        <f t="shared" si="72"/>
+        <f t="shared" si="73"/>
         <v>Genoud_etal_2018_TableS2</v>
       </c>
       <c r="L51" s="5" t="str">
-        <f t="shared" ref="L51:L52" si="79">IF(ISBLANK(I51),TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTJOIN("_", FALSE, H51, SUBSTITUTE(J51,"_", "")), "/", "%2F"), ":", "%3A"), " ", "")),TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTJOIN("_", FALSE, I51, SUBSTITUTE(J51,"_", "")), "/", "%2F"), ":", "%3A"), " ", "")))</f>
+        <f t="shared" ref="L51:L52" si="80">IF(ISBLANK(I51),TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTJOIN("_", FALSE, H51, SUBSTITUTE(J51,"_", "")), "/", "%2F"), ":", "%3A"), " ", "")),TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTJOIN("_", FALSE, I51, SUBSTITUTE(J51,"_", "")), "/", "%2F"), ":", "%3A"), " ", "")))</f>
         <v>10.1111%2Fbrv.12350_TableS2</v>
       </c>
       <c r="N51" s="5" t="s">
@@ -5466,19 +5466,19 @@
         <v>6</v>
       </c>
       <c r="C52" s="9" t="str">
-        <f t="shared" si="68"/>
+        <f t="shared" si="69"/>
         <v>Mota_etal_2019</v>
       </c>
       <c r="D52" s="9" t="str">
-        <f t="shared" si="69"/>
+        <f t="shared" si="70"/>
         <v>Mota</v>
       </c>
       <c r="E52" s="2" t="str">
-        <f t="shared" si="70"/>
+        <f t="shared" si="71"/>
         <v>etal</v>
       </c>
       <c r="F52" s="9" t="str">
-        <f t="shared" si="71"/>
+        <f t="shared" si="72"/>
         <v>2019</v>
       </c>
       <c r="G52" s="9"/>
@@ -5491,11 +5491,11 @@
         <v>272</v>
       </c>
       <c r="K52" s="5" t="str">
-        <f t="shared" si="72"/>
+        <f t="shared" si="73"/>
         <v>Mota_etal_2019_SupplementaryTableS1</v>
       </c>
       <c r="L52" s="5" t="str">
-        <f t="shared" si="79"/>
+        <f t="shared" si="80"/>
         <v>10.1073%2Fpnas.1716956116_SupplementaryTableS1</v>
       </c>
       <c r="N52" s="5" t="s">
@@ -5521,19 +5521,19 @@
         <v>9</v>
       </c>
       <c r="C53" s="9" t="str">
-        <f t="shared" si="68"/>
+        <f t="shared" si="69"/>
         <v>Burish_etal_2010</v>
       </c>
       <c r="D53" s="9" t="str">
-        <f t="shared" si="69"/>
+        <f t="shared" si="70"/>
         <v>Burish</v>
       </c>
       <c r="E53" s="2" t="str">
-        <f t="shared" si="70"/>
+        <f t="shared" si="71"/>
         <v>etal</v>
       </c>
       <c r="F53" s="9" t="str">
-        <f t="shared" ref="F53" si="80">_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(A53, "("), ")")</f>
+        <f t="shared" ref="F53" si="81">_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(A53, "("), ")")</f>
         <v>2010</v>
       </c>
       <c r="G53" s="9"/>
@@ -5546,11 +5546,11 @@
         <v>52</v>
       </c>
       <c r="K53" s="5" t="str">
-        <f t="shared" ref="K53" si="81">TRIM(_xlfn.TEXTJOIN("_",FALSE,C53,(SUBSTITUTE(SUBSTITUTE(J53," ",""), "_", ""))))</f>
+        <f t="shared" ref="K53" si="82">TRIM(_xlfn.TEXTJOIN("_",FALSE,C53,(SUBSTITUTE(SUBSTITUTE(J53," ",""), "_", ""))))</f>
         <v>Burish_etal_2010_Table1</v>
       </c>
       <c r="L53" s="5" t="str">
-        <f t="shared" ref="L53" si="82">IF(ISBLANK(I53),TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTJOIN("_", FALSE, H53, SUBSTITUTE(J53,"_", "")), "/", "%2F"), ":", "%3A"), " ", "")),TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTJOIN("_", FALSE, I53, SUBSTITUTE(J53,"_", "")), "/", "%2F"), ":", "%3A"), " ", "")))</f>
+        <f t="shared" ref="L53" si="83">IF(ISBLANK(I53),TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTJOIN("_", FALSE, H53, SUBSTITUTE(J53,"_", "")), "/", "%2F"), ":", "%3A"), " ", "")),TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTJOIN("_", FALSE, I53, SUBSTITUTE(J53,"_", "")), "/", "%2F"), ":", "%3A"), " ", "")))</f>
         <v>10.1159%2F000319019_Table1</v>
       </c>
       <c r="N53" t="s">
@@ -5588,27 +5588,27 @@
         <v>9</v>
       </c>
       <c r="C54" s="9" t="str">
-        <f t="shared" ref="C54:C59" si="83">D54 &amp; IF(E54&lt;&gt;"", "_" &amp; E54, "_") &amp; IF(F54&lt;&gt;"", "_" &amp; F54, "_") &amp; IF(G54&lt;&gt;"", "_" &amp; G54, "")</f>
+        <f t="shared" ref="C54:C59" si="84">D54 &amp; IF(E54&lt;&gt;"", "_" &amp; E54, "_") &amp; IF(F54&lt;&gt;"", "_" &amp; F54, "_") &amp; IF(G54&lt;&gt;"", "_" &amp; G54, "")</f>
         <v>Burish_etal_2010</v>
       </c>
       <c r="D54" s="9" t="str">
-        <f t="shared" ref="D54:D59" si="84">SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTBEFORE(A54,","), "-", ""), " ", "")</f>
+        <f t="shared" ref="D54:D59" si="85">SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTBEFORE(A54,","), "-", ""), " ", "")</f>
         <v>Burish</v>
       </c>
       <c r="E54" s="2" t="str">
-        <f t="shared" ref="E54:E59" si="85">IF(ISNUMBER(FIND("&amp;", A54)),
+        <f t="shared" ref="E54:E59" si="86">IF(ISNUMBER(FIND("&amp;", A54)),
     IF(LEN(A54)-LEN(SUBSTITUTE(A54, ",", ""))&gt;=6, "etal", MID(A54, SEARCH("&amp; ", A54)+2, SEARCH(",", A54, SEARCH("&amp; ", A54)+2) - SEARCH("&amp; ", A54)-2)),
     ""
 )</f>
         <v>etal</v>
       </c>
       <c r="F54" s="9" t="str">
-        <f t="shared" ref="F54:F59" si="86">_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(A54, "("), ")")</f>
+        <f t="shared" ref="F54:F59" si="87">_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(A54, "("), ")")</f>
         <v>2010</v>
       </c>
       <c r="G54" s="9"/>
       <c r="H54" t="str">
-        <f t="shared" ref="H54:H59" si="87">_xlfn.TEXTAFTER(A54,"https://doi.org/")</f>
+        <f t="shared" ref="H54:H59" si="88">_xlfn.TEXTAFTER(A54,"https://doi.org/")</f>
         <v>10.1159/000319019</v>
       </c>
       <c r="I54" s="5"/>
@@ -5616,11 +5616,11 @@
         <v>276</v>
       </c>
       <c r="K54" s="5" t="str">
-        <f t="shared" ref="K54:K55" si="88">TRIM(_xlfn.TEXTJOIN("_",FALSE,C54,(SUBSTITUTE(SUBSTITUTE(J54," ",""), "_", ""))))</f>
+        <f t="shared" ref="K54:K55" si="89">TRIM(_xlfn.TEXTJOIN("_",FALSE,C54,(SUBSTITUTE(SUBSTITUTE(J54," ",""), "_", ""))))</f>
         <v>Burish_etal_2010_SupplementaryTable1</v>
       </c>
       <c r="L54" s="5" t="str">
-        <f t="shared" ref="L54:L55" si="89">IF(ISBLANK(I54),TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTJOIN("_", FALSE, H54, SUBSTITUTE(J54,"_", "")), "/", "%2F"), ":", "%3A"), " ", "")),TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTJOIN("_", FALSE, I54, SUBSTITUTE(J54,"_", "")), "/", "%2F"), ":", "%3A"), " ", "")))</f>
+        <f t="shared" ref="L54:L55" si="90">IF(ISBLANK(I54),TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTJOIN("_", FALSE, H54, SUBSTITUTE(J54,"_", "")), "/", "%2F"), ":", "%3A"), " ", "")),TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTJOIN("_", FALSE, I54, SUBSTITUTE(J54,"_", "")), "/", "%2F"), ":", "%3A"), " ", "")))</f>
         <v>10.1159%2F000319019_SupplementaryTable1</v>
       </c>
       <c r="N54" s="5" t="s">
@@ -5655,34 +5655,34 @@
         <v>x</v>
       </c>
       <c r="C55" s="9" t="str">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>Fu_etal_2013</v>
       </c>
       <c r="D55" s="9" t="str">
-        <f t="shared" si="84"/>
+        <f t="shared" si="85"/>
         <v>Fu</v>
       </c>
       <c r="E55" s="2" t="str">
-        <f t="shared" si="85"/>
+        <f t="shared" si="86"/>
         <v>etal</v>
       </c>
       <c r="F55" s="9" t="str">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>2013</v>
       </c>
       <c r="H55" t="str">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>10.1007/s00429-012-0462-x</v>
       </c>
       <c r="J55" s="1" t="s">
         <v>52</v>
       </c>
       <c r="K55" s="5" t="str">
-        <f t="shared" si="88"/>
+        <f t="shared" si="89"/>
         <v>Fu_etal_2013_Table1</v>
       </c>
       <c r="L55" s="5" t="str">
-        <f t="shared" si="89"/>
+        <f t="shared" si="90"/>
         <v>10.1007%2Fs00429-012-0462-x_Table1</v>
       </c>
       <c r="N55" s="5" t="s">
@@ -5711,34 +5711,34 @@
         <v>5</v>
       </c>
       <c r="C56" s="9" t="str">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>MacLarnon__1996</v>
       </c>
       <c r="D56" s="9" t="str">
-        <f t="shared" si="84"/>
+        <f t="shared" si="85"/>
         <v>MacLarnon</v>
       </c>
       <c r="E56" s="2" t="str">
-        <f t="shared" si="85"/>
+        <f t="shared" si="86"/>
         <v/>
       </c>
       <c r="F56" s="9" t="str">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>1996</v>
       </c>
       <c r="H56" t="str">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>10.1006/jhev.1996.0005</v>
       </c>
       <c r="J56" s="1" t="s">
         <v>52</v>
       </c>
       <c r="K56" s="5" t="str">
-        <f t="shared" ref="K56:K59" si="90">TRIM(_xlfn.TEXTJOIN("_",FALSE,C56,(SUBSTITUTE(SUBSTITUTE(J56," ",""), "_", ""))))</f>
+        <f t="shared" ref="K56:K59" si="91">TRIM(_xlfn.TEXTJOIN("_",FALSE,C56,(SUBSTITUTE(SUBSTITUTE(J56," ",""), "_", ""))))</f>
         <v>MacLarnon__1996_Table1</v>
       </c>
       <c r="L56" s="5" t="str">
-        <f t="shared" ref="L56:L59" si="91">IF(ISBLANK(I56),TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTJOIN("_", FALSE, H56, SUBSTITUTE(J56,"_", "")), "/", "%2F"), ":", "%3A"), " ", "")),TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTJOIN("_", FALSE, I56, SUBSTITUTE(J56,"_", "")), "/", "%2F"), ":", "%3A"), " ", "")))</f>
+        <f t="shared" ref="L56:L59" si="92">IF(ISBLANK(I56),TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTJOIN("_", FALSE, H56, SUBSTITUTE(J56,"_", "")), "/", "%2F"), ":", "%3A"), " ", "")),TRIM(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(_xlfn.TEXTJOIN("_", FALSE, I56, SUBSTITUTE(J56,"_", "")), "/", "%2F"), ":", "%3A"), " ", "")))</f>
         <v>10.1006%2Fjhev.1996.0005_Table1</v>
       </c>
       <c r="N56" s="5" t="s">
@@ -5761,34 +5761,34 @@
         <v>7</v>
       </c>
       <c r="C57" s="9" t="str">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>Wimberly_etal_2021</v>
       </c>
       <c r="D57" s="9" t="str">
-        <f t="shared" si="84"/>
+        <f t="shared" si="85"/>
         <v>Wimberly</v>
       </c>
       <c r="E57" s="2" t="str">
-        <f t="shared" si="85"/>
+        <f t="shared" si="86"/>
         <v>etal</v>
       </c>
       <c r="F57" s="9" t="str">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>2021</v>
       </c>
       <c r="H57" t="str">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>10.1098/rspb.2021.0937</v>
       </c>
       <c r="J57" t="s">
         <v>338</v>
       </c>
       <c r="K57" s="5" t="str">
-        <f t="shared" si="90"/>
+        <f t="shared" si="91"/>
         <v>Wimberly_etal_2021_mammalgait.txt</v>
       </c>
       <c r="L57" s="5" t="str">
-        <f t="shared" si="91"/>
+        <f t="shared" si="92"/>
         <v>10.1098%2Frspb.2021.0937_mammalgait.txt</v>
       </c>
       <c r="N57" s="5" t="s">
@@ -5808,34 +5808,34 @@
         <v>8</v>
       </c>
       <c r="C58" s="9" t="str">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>Granatosky__2018</v>
       </c>
       <c r="D58" s="9" t="str">
-        <f t="shared" si="84"/>
+        <f t="shared" si="85"/>
         <v>Granatosky</v>
       </c>
       <c r="E58" s="2" t="str">
-        <f t="shared" si="85"/>
+        <f t="shared" si="86"/>
         <v/>
       </c>
       <c r="F58" s="9" t="str">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>2018</v>
       </c>
       <c r="H58" t="str">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>10.1111/jzo.12608</v>
       </c>
       <c r="J58" t="s">
         <v>91</v>
       </c>
       <c r="K58" s="5" t="str">
-        <f t="shared" si="90"/>
+        <f t="shared" si="91"/>
         <v>Granatosky__2018_TableS1</v>
       </c>
       <c r="L58" s="5" t="str">
-        <f t="shared" si="91"/>
+        <f t="shared" si="92"/>
         <v>10.1111%2Fjzo.12608_TableS1</v>
       </c>
       <c r="N58" s="5" t="s">
@@ -5858,34 +5858,34 @@
         <v>1</v>
       </c>
       <c r="C59" s="9" t="str">
-        <f t="shared" si="83"/>
+        <f t="shared" si="84"/>
         <v>Wilman_etal_2014</v>
       </c>
       <c r="D59" s="9" t="str">
-        <f t="shared" si="84"/>
+        <f t="shared" si="85"/>
         <v>Wilman</v>
       </c>
       <c r="E59" s="2" t="str">
-        <f t="shared" si="85"/>
+        <f t="shared" si="86"/>
         <v>etal</v>
       </c>
       <c r="F59" s="9" t="str">
-        <f t="shared" si="86"/>
+        <f t="shared" si="87"/>
         <v>2014</v>
       </c>
       <c r="H59" t="str">
-        <f t="shared" si="87"/>
+        <f t="shared" si="88"/>
         <v>10.1890/13-1917.1</v>
       </c>
       <c r="J59" t="s">
         <v>339</v>
       </c>
       <c r="K59" s="5" t="str">
-        <f t="shared" si="90"/>
+        <f t="shared" si="91"/>
         <v>Wilman_etal_2014_MamFuncDat.txt</v>
       </c>
       <c r="L59" s="5" t="str">
-        <f t="shared" si="91"/>
+        <f t="shared" si="92"/>
         <v>10.1890%2F13-1917.1_MamFuncDat.txt</v>
       </c>
       <c r="O59" t="str">
@@ -6638,15 +6638,15 @@
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED7313F8-A05E-4214-AA83-B148B6D9FF29}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
updated Baron, Andelin, Avelino-Souza
Used Claude to help with updating scripts
</commit_message>
<xml_diff>
--- a/__ReadMe.xlsx
+++ b/__ReadMe.xlsx
@@ -1,45 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30125"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://alleninstitute.sharepoint.com/sites/MammalianM1/Shared Documents/General/Species/Evo-M1-Trait-Data/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="13_ncr:1_{D1DDFD38-8A94-4545-B3F0-CD27884E4A68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FA981651-3638-4A6B-8CAB-97603806A668}"/>
   <bookViews>
-    <workbookView xWindow="-80" yWindow="660" windowWidth="34560" windowHeight="20460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-80" yWindow="660" windowWidth="34560" windowHeight="20460" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Pipeline" sheetId="3" r:id="rId2"/>
-    <sheet name="Conflicts" sheetId="4" r:id="rId3"/>
-    <sheet name="FileList" sheetId="5" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Pipeline" sheetId="3" state="visible" r:id="rId2"/>
+    <sheet name="Conflicts" sheetId="4" state="visible" r:id="rId3"/>
+    <sheet name="FileList" sheetId="5" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="805" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="481">
   <si>
     <t>Citation (APA 7th-Annotated)</t>
   </si>
@@ -1288,12 +1265,208 @@
   </si>
   <si>
     <t>README.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Files</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.0000%2Fplaceholder.1_Table1.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1002%2Fcne.24605_TABLE1.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1002%2Fcne.24605_TABLE2.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1002%2Fcne.24985_TABLE1.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1002%2Fcne.24985_TABLE2.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1002%2Fcne.25669_TABLE1.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1002%2Fcne.70089_TABLE1.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1006%2Fjhev.1996.0005_Table1.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1007%2Fs004220000205_Figure3.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1016%2Fj.jhevol.2008.08.004_Table2.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1016%2Fj.jhevol.2008.08.004_Table7.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1016%2Fj.jhevol.2008.08.004_TableS1.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1016%2Fj.jhevol.2008.08.004_TableS2.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1016%2Fj.jhevol.2008.08.004_TableS3.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1016%2Fj.jhevol.2008.08.004_Tree.nex</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1016%2Fs0166-4328(98)00151-x_Table1.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1037%2F0735-7036.115.1.29_Table1.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1037%2F0735-7036.115.1.29_Table2.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1037%2F0735-7036.115.1.29_Table3.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1037%2F0735-7036.115.1.29_Table4.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1038%2Fs41467-020-14356-3_SupplementaryData3.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1038%2Fs41598-018-26062-8_Table1.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1038%2Fs41598-018-26062-8_TableS1.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1038%2Fs41598-018-26062-8_TableS5.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1073%2Fpnas.0905777106_TableS1.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1093%2Fjmammal%2Fgyz043_SupplementaryDataSD1.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1093%2Fjmammal%2Fgyz043.ReadMe.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1093%2Foso%2F9780198568742.003.0006_Table6.1.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1098%2Frspb.2015.1853_Table1.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1126%2Fscience.aaa9101_TableS1.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1159%2F000124401_TableI.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1159%2F000319019_SupplementaryTable1.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1159%2F000319019_Table1.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1159%2F000323671_SupplementaryTable1.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1159%2F000323671_SupplementaryTable2.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1159%2F000323671.ReadMe.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1159%2F000437413_Table1.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1159%2F000437413_Table2.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1159%2F000437413_Table3.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1159%2F000437413_Table4.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1159%2F000437413_Table5.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1159%2F000452856_TableS1.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1371%2Fjournal.pbio.1002000_TableS1.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1371%2Fjournal.pbio.1002000_TableS8.ReadMe.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1371%2Fjournal.pbio.1002000_TableS8.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1523%2FJNEUROSCI.2339-19.2020_Table1.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1523%2FJNEUROSCI.2339-19.2020_unpublished.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.3389%25Ffnana.2013.00035.svg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.3389%2Ffnana.2013.00035_Figure2TopLeft.ReadMe.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.3389%2Ffnana.2013.00035_Figure2TopLeft.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.3389%2Ffnana.2013.00035_Table1-a.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.3389%2Ffnana.2013.00035_Table1-b.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.3389%2Ffnana.2013.00035.ReadMe.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.3389%2Ffnana.2017.00118_Table1.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.3389%2Ffnhum.2013.00424_TableS2partial.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.3389%2Ffnhum.2013.00424.ReadMe.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.3389%2Ffnins.2021.632853_TABLE1.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.6084%2Fm9.figshare.c.3899422.v1_Dataset1.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.7554%2FeLife.77875_Supplementaryfile3.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.7554%2FeLife.77875_Table1.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">README.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WOS%3A000225086000011_TABLE1.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Andelin_etal_2019_Table4.tsv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1093%2Fcercor%2Fbhy315_Table4.tsv</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="7">
     <font>
       <sz val="12"/>
@@ -1306,45 +1479,34 @@
       <sz val="11"/>
       <color rgb="FF3F3F76"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <color rgb="FF3F3F76"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
+      <b/>
     </font>
     <font>
-      <i/>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
-      <color rgb="FF3F3F76"/>
+      <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <i/>
     </font>
   </fonts>
   <fills count="3">
@@ -1381,7 +1543,6 @@
       <bottom style="thin">
         <color rgb="FF7F7F7F"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -1390,39 +1551,33 @@
       <right style="thin">
         <color rgb="FF7F7F7F"/>
       </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Input" xfId="1" builtinId="20"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1734,146 +1889,151 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AH83"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="42.125" customWidth="1"/>
-    <col min="2" max="2" width="5.125" customWidth="1"/>
-    <col min="3" max="3" width="22.875" customWidth="1"/>
-    <col min="4" max="4" width="34.875" customWidth="1"/>
-    <col min="5" max="5" width="2" customWidth="1"/>
-    <col min="6" max="6" width="23.625" customWidth="1"/>
-    <col min="7" max="7" width="16.875" customWidth="1"/>
-    <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="9" width="5.125" customWidth="1"/>
-    <col min="10" max="10" width="12" customWidth="1"/>
-    <col min="11" max="11" width="31.125" customWidth="1"/>
-    <col min="12" max="12" width="46.5" customWidth="1"/>
-    <col min="13" max="13" width="21.5" customWidth="1"/>
-    <col min="14" max="14" width="15.375" customWidth="1"/>
-    <col min="15" max="15" width="24" customWidth="1"/>
-    <col min="16" max="16" width="10" customWidth="1"/>
-    <col min="17" max="20" width="14.125" customWidth="1"/>
-    <col min="21" max="21" width="13.875" customWidth="1"/>
-    <col min="22" max="22" width="12.625" customWidth="1"/>
-    <col min="23" max="23" width="22.125" customWidth="1"/>
-    <col min="24" max="24" width="14.375" customWidth="1"/>
-    <col min="25" max="25" width="39.5" customWidth="1"/>
-    <col min="26" max="26" width="11.125" customWidth="1"/>
-    <col min="27" max="27" width="5" customWidth="1"/>
-    <col min="28" max="28" width="7.5" customWidth="1"/>
-    <col min="29" max="29" width="10.625" customWidth="1"/>
-    <col min="30" max="30" width="10.875" customWidth="1"/>
-    <col min="31" max="31" width="11" customWidth="1"/>
-    <col min="32" max="34" width="10.875" customWidth="1"/>
+    <col min="1" max="1" width="42.125" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="5.125" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="22.875" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="34.875" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="2" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="23.625" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="16.875" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="15" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="5.125" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="12" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="31.125" hidden="0" customWidth="1"/>
+    <col min="12" max="12" width="46.5" hidden="0" customWidth="1"/>
+    <col min="13" max="13" width="21.5" hidden="0" customWidth="1"/>
+    <col min="14" max="14" width="15.375" hidden="0" customWidth="1"/>
+    <col min="15" max="15" width="24" hidden="0" customWidth="1"/>
+    <col min="16" max="16" width="10" hidden="0" customWidth="1"/>
+    <col min="17" max="17" width="14.125" hidden="0" customWidth="1"/>
+    <col min="18" max="18" width="14.125" hidden="0" customWidth="1"/>
+    <col min="19" max="19" width="14.125" hidden="0" customWidth="1"/>
+    <col min="20" max="20" width="14.125" hidden="0" customWidth="1"/>
+    <col min="21" max="21" width="13.875" hidden="0" customWidth="1"/>
+    <col min="22" max="22" width="12.625" hidden="0" customWidth="1"/>
+    <col min="23" max="23" width="22.125" hidden="0" customWidth="1"/>
+    <col min="24" max="24" width="14.375" hidden="0" customWidth="1"/>
+    <col min="25" max="25" width="39.5" hidden="0" customWidth="1"/>
+    <col min="26" max="26" width="11.125" hidden="0" customWidth="1"/>
+    <col min="27" max="27" width="5" hidden="0" customWidth="1"/>
+    <col min="28" max="28" width="7.5" hidden="0" customWidth="1"/>
+    <col min="29" max="29" width="10.625" hidden="0" customWidth="1"/>
+    <col min="30" max="30" width="10.875" hidden="0" customWidth="1"/>
+    <col min="31" max="31" width="11" hidden="0" customWidth="1"/>
+    <col min="32" max="32" width="10.875" hidden="0" customWidth="1"/>
+    <col min="33" max="33" width="10.875" hidden="0" customWidth="1"/>
+    <col min="34" max="34" width="10.875" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" ht="15.95" customHeight="1">
-      <c r="A1" s="6" t="s">
+    <row r="1" ht="15.95" customHeight="1">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="N1" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="6" t="s">
+      <c r="O1" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="6" t="s">
+      <c r="P1" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="6" t="s">
+      <c r="Q1" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="6" t="s">
+      <c r="R1" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="6" t="s">
+      <c r="S1" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="6" t="s">
+      <c r="T1" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="6" t="s">
+      <c r="U1" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="6" t="s">
+      <c r="V1" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="6" t="s">
+      <c r="W1" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="6" t="s">
+      <c r="X1" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="6" t="s">
+      <c r="Y1" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="6" t="s">
+      <c r="Z1" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="6" t="s">
+      <c r="AA1" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="6" t="s">
+      <c r="AB1" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="6" t="s">
+      <c r="AC1" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="6" t="s">
+      <c r="AD1" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="6" t="s">
+      <c r="AE1" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="6" t="s">
+      <c r="AF1" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" s="6" t="s">
+      <c r="AG1" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" s="6" t="s">
+      <c r="AH1" s="9" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:34" ht="15.95" customHeight="1">
+    <row r="2" ht="15.95" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>34</v>
       </c>
@@ -1925,7 +2085,7 @@
       <c r="Y2" s="1"/>
       <c r="Z2" s="1"/>
     </row>
-    <row r="3" spans="1:34" ht="15.95" customHeight="1">
+    <row r="3" ht="15.95" customHeight="1">
       <c r="A3" s="1" t="s">
         <v>37</v>
       </c>
@@ -1971,17 +2131,77 @@
         <f t="array" ref="M3">IFERROR(INDEX(FileList!$A$1:$A$100, MATCH(L3, _xlfn.TEXTBEFORE(FileList!$A$1:$A$100, ".tsv"), 0)), "notfound")</f>
         <v>10.1002%2Fcne.70089_TABLE1.tsv</v>
       </c>
+      <c r="N3" s="1" t="inlineStr">
+        <is>
+          <t>xml:space="preserve"&gt;Table 1. Cellular composition of the brain of a Northern minke whale (Balaenoptera acutorostrata)</t>
+        </is>
+      </c>
+      <c r="P3" s="1" t="inlineStr">
+        <is>
+          <t>xml:space="preserve"&gt;FINISHED</t>
+        </is>
+      </c>
+      <c r="Q3" s="1" t="inlineStr">
+        <is>
+          <t>xml:space="preserve"&gt;added</t>
+        </is>
+      </c>
+      <c r="R3" s="1" t="inlineStr">
+        <is>
+          <t>xml:space="preserve"&gt;AvelinodeSouza_etal_2025_TABLE1_snapshot.csv</t>
+        </is>
+      </c>
+      <c r="S3" s="1" t="inlineStr">
+        <is>
+          <t>xml:space="preserve"&gt;Y</t>
+        </is>
+      </c>
+      <c r="T3" s="1" t="inlineStr">
+        <is>
+          <t>xml:space="preserve"&gt;AvelinodeSouza_etal_2025_TABLE1.csv</t>
+        </is>
+      </c>
+      <c r="U3" s="1" t="inlineStr">
+        <is>
+          <t>xml:space="preserve"&gt;pdf</t>
+        </is>
+      </c>
       <c r="V3" s="1" t="s">
         <v>36</v>
       </c>
+      <c r="W3" s="1" t="inlineStr">
+        <is>
+          <t>xml:space="preserve"&gt;https://onlinelibrary.wiley.com/doi/10.1002/cne.70089</t>
+        </is>
+      </c>
+      <c r="X3" s="1" t="inlineStr">
+        <is>
+          <t>xml:space="preserve"&gt;https://doi.org/10.1002/cne.70089</t>
+        </is>
+      </c>
       <c r="Y3" s="1" t="s">
         <v>39</v>
       </c>
       <c r="Z3" s="1" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="4" spans="1:34" ht="15.95" customHeight="1">
+      <c r="AA3" s="1" t="inlineStr">
+        <is>
+          <t>xml:space="preserve"&gt;HH</t>
+        </is>
+      </c>
+      <c r="AB3" s="1" t="inlineStr">
+        <is>
+          <t>xml:space="preserve"&gt;HH</t>
+        </is>
+      </c>
+      <c r="AE3" s="1" t="inlineStr">
+        <is>
+          <t>xml:space="preserve"&gt;placental mammals</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="15.95" customHeight="1">
       <c r="A4" s="1" t="s">
         <v>41</v>
       </c>
@@ -2028,10 +2248,10 @@
         <v>notfound</v>
       </c>
       <c r="V4" s="1"/>
-      <c r="Y4" s="13"/>
+      <c r="Y4" s="2"/>
       <c r="Z4" s="1"/>
     </row>
-    <row r="5" spans="1:34" ht="15.95" customHeight="1">
+    <row r="5" ht="15.95" customHeight="1">
       <c r="A5" s="1" t="s">
         <v>43</v>
       </c>
@@ -2090,7 +2310,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:34" ht="15.95" customHeight="1">
+    <row r="6" ht="15.95" customHeight="1">
       <c r="A6" s="1" t="s">
         <v>47</v>
       </c>
@@ -2149,7 +2369,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:34" ht="15.95" customHeight="1">
+    <row r="7" ht="15.95" customHeight="1">
       <c r="A7" s="1" t="s">
         <v>49</v>
       </c>
@@ -2176,7 +2396,6 @@
     IF(LEN(A7)-LEN(SUBSTITUTE(A7, ",", ""))&gt;=6, "etal", MID(A7, SEARCH("&amp; ", A7)+2, SEARCH(",", A7, SEARCH("&amp; ", A7)+2) - SEARCH("&amp; ", A7)-2)),
     ""
 )</f>
-        <v/>
       </c>
       <c r="I7" t="str">
         <f t="shared" ref="I7:I50" si="35">_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(A7, "("), ")")</f>
@@ -2199,7 +2418,7 @@
         <v>notfound</v>
       </c>
     </row>
-    <row r="8" spans="1:34" ht="17.100000000000001" customHeight="1">
+    <row r="8" ht="17.100000000000001" customHeight="1">
       <c r="A8" s="1" t="s">
         <v>52</v>
       </c>
@@ -2283,7 +2502,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="9" spans="1:34" ht="17.100000000000001" customHeight="1">
+    <row r="9" ht="17.100000000000001" customHeight="1">
       <c r="A9" s="1" t="s">
         <v>65</v>
       </c>
@@ -2345,7 +2564,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="10" spans="1:34" ht="15.95" customHeight="1">
+    <row r="10" ht="15.95" customHeight="1">
       <c r="A10" s="1" t="s">
         <v>65</v>
       </c>
@@ -2400,6 +2619,26 @@
       <c r="R10" s="1" t="s">
         <v>75</v>
       </c>
+      <c r="T10" s="1" t="inlineStr">
+        <is>
+          <t>xml:space="preserve"&gt;Burish_etal_2010_Table1.csv</t>
+        </is>
+      </c>
+      <c r="U10" s="1" t="inlineStr">
+        <is>
+          <t>xml:space="preserve"&gt;pdf</t>
+        </is>
+      </c>
+      <c r="V10" s="1" t="inlineStr">
+        <is>
+          <t>xml:space="preserve"&gt;table</t>
+        </is>
+      </c>
+      <c r="X10" s="1" t="inlineStr">
+        <is>
+          <t>xml:space="preserve"&gt;https://doi.org/10.1159/000319019</t>
+        </is>
+      </c>
       <c r="Z10" s="1" t="s">
         <v>76</v>
       </c>
@@ -2410,7 +2649,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="11" spans="1:34" ht="15.95" customHeight="1">
+    <row r="11" ht="15.95" customHeight="1">
       <c r="A11" s="1" t="s">
         <v>77</v>
       </c>
@@ -2494,7 +2733,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="12" spans="1:34" ht="15.95" customHeight="1">
+    <row r="12" ht="15.95" customHeight="1">
       <c r="A12" s="1" t="s">
         <v>77</v>
       </c>
@@ -2580,7 +2819,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="13" spans="1:34" ht="15.95" customHeight="1">
+    <row r="13" ht="15.95" customHeight="1">
       <c r="A13" s="1" t="s">
         <v>96</v>
       </c>
@@ -2601,7 +2840,6 @@
       </c>
       <c r="H13" t="str">
         <f t="shared" si="34"/>
-        <v/>
       </c>
       <c r="I13" t="str">
         <f t="shared" si="35"/>
@@ -2657,7 +2895,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="14" spans="1:34" ht="15.95" customHeight="1">
+    <row r="14" ht="15.95" customHeight="1">
       <c r="A14" s="1" t="s">
         <v>107</v>
       </c>
@@ -2744,7 +2982,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="15" spans="1:34" ht="15.95" customHeight="1">
+    <row r="15" ht="15.95" customHeight="1">
       <c r="A15" s="1" t="s">
         <v>115</v>
       </c>
@@ -2794,7 +3032,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="16" spans="1:34" ht="15.95" customHeight="1">
+    <row r="16" ht="15.95" customHeight="1">
       <c r="A16" s="1" t="s">
         <v>118</v>
       </c>
@@ -2865,7 +3103,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="17" spans="1:32" ht="15.95" customHeight="1">
+    <row r="17" ht="15.95" customHeight="1">
       <c r="A17" s="1" t="s">
         <v>118</v>
       </c>
@@ -2936,7 +3174,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="18" spans="1:32" ht="15.95" customHeight="1">
+    <row r="18" ht="15.95" customHeight="1">
       <c r="A18" s="1" t="s">
         <v>118</v>
       </c>
@@ -3007,7 +3245,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="19" spans="1:32" ht="15.95" customHeight="1">
+    <row r="19" ht="15.95" customHeight="1">
       <c r="A19" s="1" t="s">
         <v>118</v>
       </c>
@@ -3078,7 +3316,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="20" spans="1:32" ht="15.95" customHeight="1">
+    <row r="20" ht="15.95" customHeight="1">
       <c r="A20" s="1" t="s">
         <v>131</v>
       </c>
@@ -3170,7 +3408,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="21" spans="1:32" ht="15.95" customHeight="1">
+    <row r="21" ht="15.95" customHeight="1">
       <c r="A21" s="1" t="s">
         <v>143</v>
       </c>
@@ -3219,7 +3457,7 @@
       <c r="Q21" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="R21" s="4" t="s">
+      <c r="R21" s="7" t="s">
         <v>144</v>
       </c>
       <c r="S21" s="1" t="s">
@@ -3250,7 +3488,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="22" spans="1:32" ht="15.95" customHeight="1">
+    <row r="22" ht="15.95" customHeight="1">
       <c r="A22" s="1" t="s">
         <v>143</v>
       </c>
@@ -3302,7 +3540,7 @@
       <c r="Q22" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="R22" s="4" t="s">
+      <c r="R22" s="7" t="s">
         <v>144</v>
       </c>
       <c r="S22" s="1" t="s">
@@ -3317,6 +3555,11 @@
       <c r="V22" s="1" t="s">
         <v>36</v>
       </c>
+      <c r="X22" s="1" t="inlineStr">
+        <is>
+          <t>xml:space="preserve"&gt;https://doi.org/10.1523/JNEUROSCI.2339-19.2020</t>
+        </is>
+      </c>
       <c r="Y22" s="1" t="s">
         <v>139</v>
       </c>
@@ -3333,8 +3576,8 @@
         <v>148</v>
       </c>
     </row>
-    <row r="23" spans="1:32" ht="15.95" customHeight="1">
-      <c r="A23" s="3" t="s">
+    <row r="23" ht="15.95" customHeight="1">
+      <c r="A23" s="6" t="s">
         <v>150</v>
       </c>
       <c r="D23" s="1" t="s">
@@ -3382,18 +3625,18 @@
       <c r="N23" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="R23" s="4"/>
+      <c r="R23" s="7"/>
       <c r="U23" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="Y23" s="11" t="s">
+      <c r="Y23" s="3" t="s">
         <v>152</v>
       </c>
       <c r="Z23" s="1" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="24" spans="1:32" ht="15.95" customHeight="1">
+    <row r="24" ht="15.95" customHeight="1">
       <c r="A24" s="1" t="s">
         <v>153</v>
       </c>
@@ -3439,7 +3682,7 @@
       <c r="N24" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="R24" s="4"/>
+      <c r="R24" s="7"/>
       <c r="U24" s="1" t="s">
         <v>90</v>
       </c>
@@ -3447,7 +3690,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="25" spans="1:32" ht="15.95" customHeight="1">
+    <row r="25" ht="15.95" customHeight="1">
       <c r="A25" s="1" t="s">
         <v>153</v>
       </c>
@@ -3496,7 +3739,7 @@
       <c r="N25" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="R25" s="4"/>
+      <c r="R25" s="7"/>
       <c r="U25" s="1" t="s">
         <v>90</v>
       </c>
@@ -3504,7 +3747,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="26" spans="1:32" ht="15.95" customHeight="1">
+    <row r="26" ht="15.95" customHeight="1">
       <c r="A26" s="1" t="s">
         <v>157</v>
       </c>
@@ -3547,7 +3790,7 @@
         <f t="array" ref="M26">IFERROR(INDEX(FileList!$A$1:$A$100, MATCH(L26, _xlfn.TEXTBEFORE(FileList!$A$1:$A$100, ".tsv"), 0)), "notfound")</f>
         <v>10.1093%2Foso%2F9780198568742.003.0006_Table6.1.tsv</v>
       </c>
-      <c r="N26" s="5"/>
+      <c r="N26" s="8"/>
       <c r="P26" s="1" t="s">
         <v>98</v>
       </c>
@@ -3588,7 +3831,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="27" spans="1:32" ht="15.95" customHeight="1">
+    <row r="27" ht="15.95" customHeight="1">
       <c r="A27" s="1" t="s">
         <v>163</v>
       </c>
@@ -3644,7 +3887,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="28" spans="1:32" ht="15" customHeight="1">
+    <row r="28" ht="15" customHeight="1">
       <c r="A28" s="1" t="s">
         <v>167</v>
       </c>
@@ -3700,7 +3943,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="29" spans="1:32" ht="15.95" customHeight="1">
+    <row r="29" ht="15.95" customHeight="1">
       <c r="A29" s="1" t="s">
         <v>167</v>
       </c>
@@ -3756,7 +3999,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="30" spans="1:32" ht="15.95" customHeight="1">
+    <row r="30" ht="15.95" customHeight="1">
       <c r="A30" s="1" t="s">
         <v>172</v>
       </c>
@@ -3809,7 +4052,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="31" spans="1:32" ht="15.95" customHeight="1">
+    <row r="31" ht="15.95" customHeight="1">
       <c r="A31" s="1" t="s">
         <v>175</v>
       </c>
@@ -3830,7 +4073,6 @@
       </c>
       <c r="H31" t="str">
         <f t="shared" si="34"/>
-        <v/>
       </c>
       <c r="I31" t="str">
         <f t="shared" si="35"/>
@@ -3859,7 +4101,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="32" spans="1:32" ht="15.95" customHeight="1">
+    <row r="32" ht="15.95" customHeight="1">
       <c r="A32" s="1" t="s">
         <v>177</v>
       </c>
@@ -3903,10 +4145,10 @@
         <f t="array" ref="M32">IFERROR(INDEX(FileList!$A$1:$A$100, MATCH(L32, _xlfn.TEXTBEFORE(FileList!$A$1:$A$100, ".tsv"), 0)), "notfound")</f>
         <v>notfound</v>
       </c>
-      <c r="N32" s="10"/>
+      <c r="N32" s="2"/>
       <c r="P32" s="1"/>
     </row>
-    <row r="33" spans="1:33" ht="15.95" customHeight="1">
+    <row r="33" ht="15.95" customHeight="1">
       <c r="A33" s="1" t="s">
         <v>178</v>
       </c>
@@ -3986,7 +4228,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="34" spans="1:33" ht="15.95" customHeight="1">
+    <row r="34" ht="15.95" customHeight="1">
       <c r="A34" s="1" t="s">
         <v>185</v>
       </c>
@@ -4035,7 +4277,7 @@
       <c r="Q34" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="R34" s="4"/>
+      <c r="R34" s="7"/>
       <c r="T34" s="1" t="str">
         <f>IF(S34="N", R34, "write file name")</f>
         <v>write file name</v>
@@ -4059,11 +4301,11 @@
         <v>186</v>
       </c>
     </row>
-    <row r="35" spans="1:33" ht="15.95" customHeight="1">
+    <row r="35" ht="15.95" customHeight="1">
       <c r="A35" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="C35" s="12" t="s">
+      <c r="C35" s="4" t="s">
         <v>188</v>
       </c>
       <c r="D35" s="1" t="s">
@@ -4108,23 +4350,23 @@
         <f t="array" ref="M35">IFERROR(INDEX(FileList!$A$1:$A$100, MATCH(L35, _xlfn.TEXTBEFORE(FileList!$A$1:$A$100, ".tsv"), 0)), "notfound")</f>
         <v>notfound</v>
       </c>
-      <c r="N35" s="10" t="s">
+      <c r="N35" s="2" t="s">
         <v>189</v>
       </c>
       <c r="P35" s="1"/>
       <c r="Q35" s="1"/>
-      <c r="R35" s="4"/>
+      <c r="R35" s="7"/>
       <c r="T35" s="1"/>
       <c r="U35" s="1"/>
       <c r="V35" s="1"/>
-      <c r="W35" s="10"/>
+      <c r="W35" s="2"/>
       <c r="Y35" s="1" t="s">
         <v>190</v>
       </c>
       <c r="AE35" s="1"/>
-      <c r="AG35" s="10"/>
-    </row>
-    <row r="36" spans="1:33" ht="15.95" customHeight="1">
+      <c r="AG35" s="2"/>
+    </row>
+    <row r="36" ht="15.95" customHeight="1">
       <c r="A36" s="1" t="s">
         <v>191</v>
       </c>
@@ -4173,7 +4415,7 @@
       <c r="Q36" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="R36" s="4"/>
+      <c r="R36" s="7"/>
       <c r="T36" s="1" t="str">
         <f>IF(S36="N", R36, "write file name")</f>
         <v>write file name</v>
@@ -4191,7 +4433,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="37" spans="1:33" ht="15.95" customHeight="1">
+    <row r="37" ht="15.95" customHeight="1">
       <c r="A37" s="1" t="s">
         <v>193</v>
       </c>
@@ -4212,7 +4454,6 @@
       </c>
       <c r="H37" t="str">
         <f t="shared" si="34"/>
-        <v/>
       </c>
       <c r="I37" t="str">
         <f t="shared" si="35"/>
@@ -4235,17 +4476,17 @@
         <v>10.1098%2Frspb.2015.1853_Table1.tsv</v>
       </c>
       <c r="N37" s="1"/>
-      <c r="R37" s="4"/>
-      <c r="U37" s="10" t="s">
+      <c r="R37" s="7"/>
+      <c r="U37" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="V37" s="10" t="s">
+      <c r="V37" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="Y37" s="10"/>
-      <c r="Z37" s="10"/>
-    </row>
-    <row r="38" spans="1:33" ht="15.95" customHeight="1">
+      <c r="Y37" s="2"/>
+      <c r="Z37" s="2"/>
+    </row>
+    <row r="38" ht="15.95" customHeight="1">
       <c r="A38" s="1" t="s">
         <v>193</v>
       </c>
@@ -4269,7 +4510,6 @@
     IF(LEN(A38)-LEN(SUBSTITUTE(A38, ",", ""))&gt;=6, "etal", MID(A38, SEARCH("&amp; ", A38)+2, SEARCH(",", A38, SEARCH("&amp; ", A38)+2) - SEARCH("&amp; ", A38)-2)),
     ""
 )</f>
-        <v/>
       </c>
       <c r="I38" t="str">
         <f t="shared" ref="I38" si="90">_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(A38, "("), ")")</f>
@@ -4294,21 +4534,21 @@
       <c r="N38" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="R38" s="4"/>
-      <c r="U38" s="10" t="s">
+      <c r="R38" s="7"/>
+      <c r="U38" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="V38" s="10" t="s">
+      <c r="V38" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="Y38" s="10" t="s">
+      <c r="Y38" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="Z38" s="10" t="s">
+      <c r="Z38" s="2" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="39" spans="1:33" ht="15.95" customHeight="1">
+    <row r="39" ht="15.95" customHeight="1">
       <c r="A39" s="1" t="s">
         <v>197</v>
       </c>
@@ -4355,7 +4595,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="40" spans="1:33" ht="18.95" customHeight="1">
+    <row r="40" ht="18.95" customHeight="1">
       <c r="A40" s="1" t="s">
         <v>197</v>
       </c>
@@ -4402,7 +4642,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="41" spans="1:33" ht="17.100000000000001" customHeight="1">
+    <row r="41" ht="17.100000000000001" customHeight="1">
       <c r="A41" s="1" t="s">
         <v>197</v>
       </c>
@@ -4449,7 +4689,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="42" spans="1:33" ht="17.100000000000001" customHeight="1">
+    <row r="42" ht="17.100000000000001" customHeight="1">
       <c r="A42" s="1" t="s">
         <v>201</v>
       </c>
@@ -4501,7 +4741,7 @@
       <c r="Q42" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="R42" s="4" t="s">
+      <c r="R42" s="7" t="s">
         <v>203</v>
       </c>
       <c r="S42" s="1" t="s">
@@ -4535,7 +4775,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="43" spans="1:33" ht="17.100000000000001" customHeight="1">
+    <row r="43" ht="17.100000000000001" customHeight="1">
       <c r="A43" s="1" t="s">
         <v>201</v>
       </c>
@@ -4587,7 +4827,7 @@
       <c r="Q43" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="R43" s="4" t="s">
+      <c r="R43" s="7" t="s">
         <v>208</v>
       </c>
       <c r="S43" s="1" t="s">
@@ -4621,7 +4861,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="44" spans="1:33" ht="17.100000000000001" customHeight="1">
+    <row r="44" ht="17.100000000000001" customHeight="1">
       <c r="A44" s="1" t="s">
         <v>201</v>
       </c>
@@ -4673,7 +4913,7 @@
       <c r="Q44" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="R44" s="4" t="s">
+      <c r="R44" s="7" t="s">
         <v>212</v>
       </c>
       <c r="S44" s="1" t="s">
@@ -4707,7 +4947,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="45" spans="1:33" ht="15.95" customHeight="1">
+    <row r="45" ht="15.95" customHeight="1">
       <c r="A45" s="1" t="s">
         <v>201</v>
       </c>
@@ -4759,7 +4999,7 @@
       <c r="Q45" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="R45" s="4" t="s">
+      <c r="R45" s="7" t="s">
         <v>215</v>
       </c>
       <c r="S45" s="1" t="s">
@@ -4793,7 +5033,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="46" spans="1:33" ht="15.95" customHeight="1">
+    <row r="46" ht="15.95" customHeight="1">
       <c r="A46" s="1" t="s">
         <v>201</v>
       </c>
@@ -4845,7 +5085,7 @@
       <c r="Q46" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="R46" s="4" t="s">
+      <c r="R46" s="7" t="s">
         <v>219</v>
       </c>
       <c r="S46" s="1" t="s">
@@ -4879,7 +5119,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="47" spans="1:33" ht="15.95" customHeight="1">
+    <row r="47" ht="15.95" customHeight="1">
       <c r="A47" s="1" t="s">
         <v>221</v>
       </c>
@@ -4931,7 +5171,7 @@
       <c r="Q47" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="R47" s="4" t="s">
+      <c r="R47" s="7" t="s">
         <v>223</v>
       </c>
       <c r="S47" s="1" t="s">
@@ -4949,6 +5189,11 @@
       <c r="W47" s="1" t="s">
         <v>103</v>
       </c>
+      <c r="X47" s="1" t="inlineStr">
+        <is>
+          <t>xml:space="preserve"&gt;https://doi.org/10.1002/cne.24985</t>
+        </is>
+      </c>
       <c r="Y47" s="1" t="s">
         <v>225</v>
       </c>
@@ -4962,7 +5207,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="48" spans="1:33" ht="15.95" customHeight="1">
+    <row r="48" ht="15.95" customHeight="1">
       <c r="A48" s="1" t="s">
         <v>221</v>
       </c>
@@ -5014,7 +5259,7 @@
       <c r="Q48" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="R48" s="4" t="s">
+      <c r="R48" s="7" t="s">
         <v>228</v>
       </c>
       <c r="S48" s="1" t="s">
@@ -5032,6 +5277,11 @@
       <c r="W48" s="1" t="s">
         <v>103</v>
       </c>
+      <c r="X48" s="1" t="inlineStr">
+        <is>
+          <t>xml:space="preserve"&gt;https://doi.org/10.1002/cne.24985</t>
+        </is>
+      </c>
       <c r="Y48" s="1" t="s">
         <v>230</v>
       </c>
@@ -5045,7 +5295,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="49" spans="1:31" ht="15.95" customHeight="1">
+    <row r="49" ht="15.95" customHeight="1">
       <c r="A49" s="1" t="s">
         <v>231</v>
       </c>
@@ -5092,7 +5342,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="50" spans="1:31" ht="15.95" customHeight="1">
+    <row r="50" ht="15.95" customHeight="1">
       <c r="A50" s="1" t="s">
         <v>231</v>
       </c>
@@ -5139,7 +5389,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="51" spans="1:31" ht="15.95" customHeight="1">
+    <row r="51" ht="15.95" customHeight="1">
       <c r="A51" s="1" t="s">
         <v>231</v>
       </c>
@@ -5189,7 +5439,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="52" spans="1:31" ht="15.95" customHeight="1">
+    <row r="52" ht="15.95" customHeight="1">
       <c r="A52" s="1" t="s">
         <v>231</v>
       </c>
@@ -5236,7 +5486,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="53" spans="1:31" ht="15.95" customHeight="1">
+    <row r="53" ht="15.95" customHeight="1">
       <c r="A53" s="1" t="s">
         <v>231</v>
       </c>
@@ -5283,7 +5533,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="54" spans="1:31" ht="15.95" customHeight="1">
+    <row r="54" ht="15.95" customHeight="1">
       <c r="A54" s="1" t="s">
         <v>231</v>
       </c>
@@ -5330,7 +5580,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="55" spans="1:31" ht="15.95" customHeight="1">
+    <row r="55" ht="15.95" customHeight="1">
       <c r="A55" s="1" t="s">
         <v>235</v>
       </c>
@@ -5386,7 +5636,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="56" spans="1:31" ht="15.95" customHeight="1">
+    <row r="56" ht="15.95" customHeight="1">
       <c r="A56" s="1" t="s">
         <v>235</v>
       </c>
@@ -5442,7 +5692,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="57" spans="1:31" ht="15.95" customHeight="1">
+    <row r="57" ht="15.95" customHeight="1">
       <c r="A57" s="1" t="s">
         <v>239</v>
       </c>
@@ -5494,7 +5744,7 @@
       <c r="Q57" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="R57" s="4"/>
+      <c r="R57" s="7"/>
       <c r="T57" s="1" t="str">
         <f>IF(S57="N", R57, "write file name")</f>
         <v>write file name</v>
@@ -5512,7 +5762,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="58" spans="1:31" ht="15.95" customHeight="1">
+    <row r="58" ht="15.95" customHeight="1">
       <c r="A58" s="1" t="s">
         <v>239</v>
       </c>
@@ -5564,7 +5814,7 @@
       <c r="Q58" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="R58" s="4"/>
+      <c r="R58" s="7"/>
       <c r="T58" s="1" t="str">
         <f>IF(S58="N", R58, "write file name")</f>
         <v>write file name</v>
@@ -5582,7 +5832,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="59" spans="1:31" ht="15.95" customHeight="1">
+    <row r="59" ht="15.95" customHeight="1">
       <c r="A59" s="1" t="s">
         <v>239</v>
       </c>
@@ -5634,7 +5884,7 @@
       <c r="Q59" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="R59" s="4"/>
+      <c r="R59" s="7"/>
       <c r="T59" s="1" t="str">
         <f>IF(S59="N", R59, "write file name")</f>
         <v>write file name</v>
@@ -5652,7 +5902,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="60" spans="1:31" ht="15.95" customHeight="1">
+    <row r="60" ht="15.95" customHeight="1">
       <c r="A60" s="1" t="s">
         <v>239</v>
       </c>
@@ -5704,7 +5954,7 @@
       <c r="Q60" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="R60" s="4"/>
+      <c r="R60" s="7"/>
       <c r="T60" s="1" t="str">
         <f>IF(S60="N", R60, "write file name")</f>
         <v>write file name</v>
@@ -5722,7 +5972,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="61" spans="1:31" ht="15.95" customHeight="1">
+    <row r="61" ht="15.95" customHeight="1">
       <c r="A61" s="1" t="s">
         <v>247</v>
       </c>
@@ -5774,7 +6024,7 @@
       <c r="Q61" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="R61" s="4" t="s">
+      <c r="R61" s="7" t="s">
         <v>249</v>
       </c>
       <c r="S61" s="1" t="s">
@@ -5811,7 +6061,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="62" spans="1:31" ht="15.95" customHeight="1">
+    <row r="62" ht="15.95" customHeight="1">
       <c r="A62" s="1" t="s">
         <v>253</v>
       </c>
@@ -5860,24 +6110,24 @@
       <c r="N62" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="P62" s="10"/>
-      <c r="Q62" s="10"/>
-      <c r="R62" s="4"/>
-      <c r="S62" s="10"/>
-      <c r="T62" s="10"/>
+      <c r="P62" s="2"/>
+      <c r="Q62" s="2"/>
+      <c r="R62" s="7"/>
+      <c r="S62" s="2"/>
+      <c r="T62" s="2"/>
       <c r="U62" s="1"/>
       <c r="V62" s="1"/>
       <c r="W62" s="1"/>
-      <c r="X62" s="10"/>
+      <c r="X62" s="2"/>
       <c r="Y62" s="1" t="s">
         <v>255</v>
       </c>
       <c r="Z62" s="1"/>
-      <c r="AA62" s="10"/>
-      <c r="AB62" s="10"/>
-      <c r="AE62" s="10"/>
-    </row>
-    <row r="63" spans="1:31" ht="15.95" customHeight="1">
+      <c r="AA62" s="2"/>
+      <c r="AB62" s="2"/>
+      <c r="AE62" s="2"/>
+    </row>
+    <row r="63" ht="15.95" customHeight="1">
       <c r="A63" s="1" t="s">
         <v>256</v>
       </c>
@@ -5923,7 +6173,7 @@
       <c r="N63" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="R63" s="4"/>
+      <c r="R63" s="7"/>
       <c r="U63" s="1" t="s">
         <v>90</v>
       </c>
@@ -5940,7 +6190,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="64" spans="1:31" ht="15.95" customHeight="1">
+    <row r="64" ht="15.95" customHeight="1">
       <c r="A64" s="1" t="s">
         <v>259</v>
       </c>
@@ -5992,7 +6242,7 @@
       <c r="Q64" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="R64" s="4" t="s">
+      <c r="R64" s="7" t="s">
         <v>261</v>
       </c>
       <c r="S64" s="1" t="s">
@@ -6020,7 +6270,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="65" spans="1:31" ht="15.95" customHeight="1">
+    <row r="65" ht="15.95" customHeight="1">
       <c r="A65" s="1" t="s">
         <v>259</v>
       </c>
@@ -6072,7 +6322,7 @@
       <c r="Q65" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="R65" s="4" t="s">
+      <c r="R65" s="7" t="s">
         <v>267</v>
       </c>
       <c r="S65" s="1" t="s">
@@ -6099,6 +6349,11 @@
       <c r="Z65" s="1" t="s">
         <v>269</v>
       </c>
+      <c r="AA65" s="1" t="inlineStr">
+        <is>
+          <t>xml:space="preserve"&gt;Kverkova</t>
+        </is>
+      </c>
       <c r="AB65" s="1" t="s">
         <v>140</v>
       </c>
@@ -6106,7 +6361,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="66" spans="1:31" ht="15.95" customHeight="1">
+    <row r="66" ht="15.95" customHeight="1">
       <c r="A66" s="1" t="s">
         <v>259</v>
       </c>
@@ -6158,7 +6413,7 @@
       <c r="Q66" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="R66" s="4" t="s">
+      <c r="R66" s="7" t="s">
         <v>272</v>
       </c>
       <c r="S66" s="1" t="s">
@@ -6185,6 +6440,11 @@
       <c r="Z66" s="1" t="s">
         <v>40</v>
       </c>
+      <c r="AA66" s="1" t="inlineStr">
+        <is>
+          <t>xml:space="preserve"&gt;Kverkova</t>
+        </is>
+      </c>
       <c r="AB66" s="1" t="s">
         <v>140</v>
       </c>
@@ -6192,7 +6452,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="67" spans="1:31" ht="15.95" customHeight="1">
+    <row r="67" ht="15.95" customHeight="1">
       <c r="A67" s="1" t="s">
         <v>275</v>
       </c>
@@ -6242,7 +6502,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="68" spans="1:31" ht="15.95" customHeight="1">
+    <row r="68" ht="15.95" customHeight="1">
       <c r="A68" s="1" t="s">
         <v>278</v>
       </c>
@@ -6295,7 +6555,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="69" spans="1:31" ht="15.95" customHeight="1">
+    <row r="69" ht="15.95" customHeight="1">
       <c r="A69" s="1" t="s">
         <v>278</v>
       </c>
@@ -6348,7 +6608,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="70" spans="1:31" ht="15.75" customHeight="1">
+    <row r="70" ht="15.75" customHeight="1">
       <c r="A70" s="1" t="s">
         <v>282</v>
       </c>
@@ -6369,7 +6629,6 @@
       </c>
       <c r="H70" t="str">
         <f t="shared" si="94"/>
-        <v/>
       </c>
       <c r="I70" t="str">
         <f t="shared" si="95"/>
@@ -6398,7 +6657,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="71" spans="1:31" ht="15.75" customHeight="1">
+    <row r="71" ht="15.75" customHeight="1">
       <c r="A71" s="1" t="s">
         <v>284</v>
       </c>
@@ -6419,7 +6678,6 @@
       </c>
       <c r="H71" t="str">
         <f t="shared" si="94"/>
-        <v/>
       </c>
       <c r="I71" t="str">
         <f t="shared" si="95"/>
@@ -6447,7 +6705,7 @@
       <c r="Q71" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="R71" s="4"/>
+      <c r="R71" s="7"/>
       <c r="T71" s="1" t="str">
         <f>IF(S71="N", R71, "write file name")</f>
         <v>write file name</v>
@@ -6477,7 +6735,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="72" spans="1:31" ht="15.75" customHeight="1">
+    <row r="72" ht="15.75" customHeight="1">
       <c r="A72" s="1" t="s">
         <v>290</v>
       </c>
@@ -6524,7 +6782,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="73" spans="1:31" ht="15.75" customHeight="1">
+    <row r="73" ht="15.75" customHeight="1">
       <c r="A73" s="1" t="s">
         <v>291</v>
       </c>
@@ -6577,7 +6835,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="74" spans="1:31" ht="15.75" customHeight="1">
+    <row r="74" ht="15.75" customHeight="1">
       <c r="A74" s="1" t="s">
         <v>295</v>
       </c>
@@ -6629,7 +6887,7 @@
       <c r="Q74" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="R74" s="4"/>
+      <c r="R74" s="7"/>
       <c r="T74" s="1" t="str">
         <f>IF(S74="N", R74, "write file name")</f>
         <v>write file name</v>
@@ -6659,7 +6917,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="75" spans="1:31" ht="15.75" customHeight="1">
+    <row r="75" ht="15.75" customHeight="1">
       <c r="A75" s="1" t="s">
         <v>300</v>
       </c>
@@ -6714,7 +6972,7 @@
       <c r="Q75" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="R75" s="4"/>
+      <c r="R75" s="7"/>
       <c r="T75" s="1" t="str">
         <f>IF(S75="N", R75, "write file name")</f>
         <v>write file name</v>
@@ -6735,7 +6993,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="76" spans="1:31" ht="15.75" customHeight="1">
+    <row r="76" ht="15.75" customHeight="1">
       <c r="A76" s="1" t="s">
         <v>300</v>
       </c>
@@ -6790,7 +7048,7 @@
       <c r="Q76" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="R76" s="4"/>
+      <c r="R76" s="7"/>
       <c r="T76" s="1" t="str">
         <f>IF(S76="N", R76, "write file name")</f>
         <v>write file name</v>
@@ -6811,7 +7069,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="77" spans="1:31" ht="15.75" customHeight="1">
+    <row r="77" ht="15.75" customHeight="1">
       <c r="A77" s="1" t="s">
         <v>306</v>
       </c>
@@ -6858,7 +7116,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="78" spans="1:31" ht="15.75" customHeight="1">
+    <row r="78" ht="15.75" customHeight="1">
       <c r="A78" s="1" t="s">
         <v>306</v>
       </c>
@@ -6905,7 +7163,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="79" spans="1:31" ht="15.75" customHeight="1">
+    <row r="79" ht="15.75" customHeight="1">
       <c r="A79" s="1" t="s">
         <v>309</v>
       </c>
@@ -6955,7 +7213,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="80" spans="1:31" ht="15.75" customHeight="1">
+    <row r="80" ht="15.75" customHeight="1">
       <c r="A80" s="1" t="s">
         <v>312</v>
       </c>
@@ -6999,7 +7257,7 @@
         <v>notfound</v>
       </c>
     </row>
-    <row r="81" spans="1:31" ht="15.75" customHeight="1">
+    <row r="81" ht="15.75" customHeight="1">
       <c r="A81" s="1" t="s">
         <v>314</v>
       </c>
@@ -7046,7 +7304,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="82" spans="1:31">
+    <row r="82">
       <c r="A82" s="1" t="s">
         <v>316</v>
       </c>
@@ -7095,7 +7353,7 @@
       <c r="Q82" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="R82" s="4"/>
+      <c r="R82" s="7"/>
       <c r="T82" s="1" t="str">
         <f>IF(S82="N", R82, "write file name")</f>
         <v>write file name</v>
@@ -7113,7 +7371,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="83" spans="1:31">
+    <row r="83">
       <c r="A83" s="1" t="s">
         <v>320</v>
       </c>
@@ -7162,7 +7420,7 @@
       <c r="Q83" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="R83" s="4"/>
+      <c r="R83" s="7"/>
       <c r="T83" s="1" t="str">
         <f>IF(S83="N", R83, "write file name")</f>
         <v>write file name</v>
@@ -7185,20 +7443,20 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="X12" r:id="rId1" display="https://elifesciences.org/download/aHR0cHM6Ly9jZG4uZWxpZmVzY2llbmNlcy5vcmcvYXJ0aWNsZXMvNzc4NzUvZWxpZmUtNzc4NzUtdjEucGRmP2Nhbm9uaWNhbFVyaT1odHRwczovL2VsaWZlc2NpZW5jZXMub3JnL2FydGljbGVzLzc3ODc1/elife-77875-v1.pdf?_hash=NStjcL9fTlmy3AQDwSiM0YgMVB3UYjO8nDg0UbwN5gM%3D" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="X11" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="X14" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="X20" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="X26" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="X71" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="X74" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="X42" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="X31:X36" r:id="rId9" display="https://karger.com/bbe/article-pdf/86/3-4/145/2264694/000437413.pdf" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="X66" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="X65" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="X61" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="X28" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="X29" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="X12" r:id="rId1h" display="https://elifesciences.org/download/aHR0cHM6Ly9jZG4uZWxpZmVzY2llbmNlcy5vcmcvYXJ0aWNsZXMvNzc4NzUvZWxpZmUtNzc4NzUtdjEucGRmP2Nhbm9uaWNhbFVyaT1odHRwczovL2VsaWZlc2NpZW5jZXMub3JnL2FydGljbGVzLzc3ODc1/elife-77875-v1.pdf?_hash=NStjcL9fTlmy3AQDwSiM0YgMVB3UYjO8nDg0UbwN5gM%3D"/>
+    <hyperlink ref="X11" r:id="rId2h"/>
+    <hyperlink ref="X14" r:id="rId3h"/>
+    <hyperlink ref="X20" r:id="rId4h"/>
+    <hyperlink ref="X26" r:id="rId5h"/>
+    <hyperlink ref="X71" r:id="rId6h"/>
+    <hyperlink ref="X74" r:id="rId7h"/>
+    <hyperlink ref="X42" r:id="rId8h"/>
+    <hyperlink ref="X31:X36" r:id="rId9h" display="https://karger.com/bbe/article-pdf/86/3-4/145/2264694/000437413.pdf"/>
+    <hyperlink ref="X66" r:id="rId10h"/>
+    <hyperlink ref="X65" r:id="rId11h"/>
+    <hyperlink ref="X61" r:id="rId12h"/>
+    <hyperlink ref="X28" r:id="rId13h"/>
+    <hyperlink ref="X29" r:id="rId14h"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -7206,105 +7464,105 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B13"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="26.125" customWidth="1"/>
+    <col min="1" max="1" width="26.125" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1">
       <c r="A1" t="s">
         <v>322</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2">
       <c r="A2" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
-      <c r="A3" s="7" t="s">
+    <row r="3">
+      <c r="A3" s="10" t="s">
         <v>324</v>
       </c>
       <c r="B3" t="s">
         <v>325</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
-      <c r="A4" s="7" t="s">
+    <row r="4">
+      <c r="A4" s="10" t="s">
         <v>326</v>
       </c>
       <c r="B4" t="s">
         <v>327</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
-      <c r="A5" s="7" t="s">
+    <row r="5">
+      <c r="A5" s="10" t="s">
         <v>328</v>
       </c>
       <c r="B5" t="s">
         <v>329</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
-      <c r="A6" s="7" t="s">
+    <row r="6">
+      <c r="A6" s="10" t="s">
         <v>330</v>
       </c>
       <c r="B6" t="s">
         <v>331</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
-      <c r="A7" s="7" t="s">
+    <row r="7">
+      <c r="A7" s="10" t="s">
         <v>332</v>
       </c>
       <c r="B7" t="s">
         <v>333</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
-      <c r="A8" s="7" t="s">
+    <row r="8">
+      <c r="A8" s="10" t="s">
         <v>334</v>
       </c>
       <c r="B8" t="s">
         <v>335</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
-      <c r="A9" s="7" t="s">
+    <row r="9">
+      <c r="A9" s="10" t="s">
         <v>336</v>
       </c>
       <c r="B9" t="s">
         <v>337</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
-      <c r="A10" s="7" t="s">
+    <row r="10">
+      <c r="A10" s="10" t="s">
         <v>338</v>
       </c>
       <c r="B10" t="s">
         <v>339</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
-      <c r="A11" s="7" t="s">
+    <row r="11">
+      <c r="A11" s="10" t="s">
         <v>340</v>
       </c>
       <c r="B11" t="s">
         <v>341</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="17.100000000000001" customHeight="1">
-      <c r="A12" s="9" t="s">
+    <row r="12" ht="17.100000000000001" customHeight="1">
+      <c r="A12" s="12" t="s">
         <v>342</v>
       </c>
       <c r="B12" t="s">
         <v>343</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
-      <c r="A13" s="8" t="s">
+    <row r="13">
+      <c r="A13" s="11" t="s">
         <v>344</v>
       </c>
     </row>
@@ -7315,26 +7573,26 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="1.875" customWidth="1"/>
-    <col min="2" max="2" width="126" customWidth="1"/>
+    <col min="1" max="1" width="1.875" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="126" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1">
       <c r="A1" t="s">
         <v>345</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2">
       <c r="C2" t="s">
         <v>346</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
-      <c r="A3">
+    <row r="3">
+      <c r="A3" t="n">
         <v>1</v>
       </c>
       <c r="B3" t="s">
@@ -7344,8 +7602,8 @@
         <v>348</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
-      <c r="A4">
+    <row r="4">
+      <c r="A4" t="n">
         <v>2</v>
       </c>
       <c r="B4" t="s">
@@ -7355,8 +7613,8 @@
         <v>350</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
-      <c r="A5">
+    <row r="5">
+      <c r="A5" t="n">
         <v>3</v>
       </c>
       <c r="B5" t="s">
@@ -7366,8 +7624,8 @@
         <v>352</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
-      <c r="A6">
+    <row r="6">
+      <c r="A6" t="n">
         <v>4</v>
       </c>
       <c r="B6" t="s">
@@ -7384,318 +7642,333 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:A61"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1">
       <c r="A1" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="s">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="3">
       <c r="A3" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="4">
       <c r="A4" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="5">
       <c r="A5" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="6">
       <c r="A6" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="7">
       <c r="A7" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="8">
       <c r="A8" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="9">
       <c r="A9" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="10">
       <c r="A10" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="11">
       <c r="A11" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="12">
       <c r="A12" t="s">
-        <v>366</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="13">
       <c r="A13" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="14">
       <c r="A14" t="s">
-        <v>368</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="15">
       <c r="A15" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="16">
       <c r="A16" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="17">
       <c r="A17" t="s">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="18">
       <c r="A18" t="s">
-        <v>372</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="19">
       <c r="A19" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="20">
       <c r="A20" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="21">
       <c r="A21" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="22">
       <c r="A22" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="23">
       <c r="A23" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="24">
       <c r="A24" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="25">
       <c r="A25" t="s">
-        <v>379</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="26">
       <c r="A26" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="27">
       <c r="A27" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="28">
       <c r="A28" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="29">
       <c r="A29" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="30">
       <c r="A30" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="31">
       <c r="A31" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="32">
       <c r="A32" t="s">
-        <v>386</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="33">
       <c r="A33" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="34">
       <c r="A34" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="35">
       <c r="A35" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="36">
       <c r="A36" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="37">
       <c r="A37" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="38">
       <c r="A38" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="39">
       <c r="A39" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="40">
       <c r="A40" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="41" spans="1:1">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="41">
       <c r="A41" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="42" spans="1:1">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="42">
       <c r="A42" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="43" spans="1:1">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="43">
       <c r="A43" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="44" spans="1:1">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="44">
       <c r="A44" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="45" spans="1:1">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="45">
       <c r="A45" t="s">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="46" spans="1:1">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="46">
       <c r="A46" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="47" spans="1:1">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="47">
       <c r="A47" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="48" spans="1:1">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="48">
       <c r="A48" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="49" spans="1:1">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="49">
       <c r="A49" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="50" spans="1:1">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="50">
       <c r="A50" t="s">
-        <v>404</v>
-      </c>
-    </row>
-    <row r="51" spans="1:1">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="51">
       <c r="A51" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="52" spans="1:1">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="52">
       <c r="A52" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="53" spans="1:1">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="53">
       <c r="A53" t="s">
-        <v>407</v>
-      </c>
-    </row>
-    <row r="54" spans="1:1">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="54">
       <c r="A54" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="55" spans="1:1">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="55">
       <c r="A55" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="56" spans="1:1">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="56">
       <c r="A56" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="57" spans="1:1">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="57">
       <c r="A57" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="58" spans="1:1">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="58">
       <c r="A58" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="59" spans="1:1">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="59">
       <c r="A59" t="s">
-        <v>413</v>
-      </c>
-    </row>
-    <row r="60" spans="1:1">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="60">
       <c r="A60" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="61" spans="1:1">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="61">
       <c r="A61" t="s">
-        <v>415</v>
+        <v>475</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s">
+        <v>478</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -7975,13 +8248,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{393CEB05-6A9C-454A-BDDF-E9F23897B6BF}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F3175246-AD22-47A4-A702-60D9C2849160}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{05209338-5D48-4750-BEDF-5F912B2D3EB2}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AF41B972-5A98-4727-887F-6AF19ECD88DB}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C092463B-DEE0-4311-BA63-23860C1DD18C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C345D4DD-977A-400F-B0B3-D8636C363C95}"/>
 </file>
</xml_diff>

<commit_message>
WIP: preserve staged repository cleanup and data updates
</commit_message>
<xml_diff>
--- a/__ReadMe.xlsx
+++ b/__ReadMe.xlsx
@@ -7116,8 +7116,10 @@
       <c r="A19" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="D19" s="3" t="s">
-        <v>102</v>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>viaDeCasien2019</t>
+        </is>
       </c>
       <c r="E19" s="2" t="str">
         <f t="shared" si="0"/>
@@ -7145,11 +7147,11 @@
       </c>
       <c r="K19" s="2" t="str">
         <f t="shared" si="6"/>
-        <v>Barks_etal_2014_unpublishedviaDeCasien</v>
+        <v>Barks_etal_2014_viaDeCasien2019</v>
       </c>
       <c r="L19" s="2" t="str">
         <f t="shared" si="7"/>
-        <v>10.1002%2Fajpa.22646_unpublishedviaDeCasien</v>
+        <v>10.1002%2Fajpa.22646_viaDeCasien2019</v>
       </c>
       <c r="M19" s="2" t="str">
         <f t="array" ref="M19">IFERROR(INDEX(AUTO_Public_TSV_FileList!$A$1:$A$1000,MATCH(TRUE(),EXACT(L19,IFERROR(_xlfn.TEXTBEFORE(AUTO_Public_TSV_FileList!$A$1:$A$1000,".tsv"),"")),0)),"notfound")</f>
@@ -7157,6 +7159,21 @@
       </c>
       <c r="O19" s="3" t="s">
         <v>103</v>
+      </c>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t>Regional volumes measured by the Sherwood / Barks teams and published in DeCasien &amp; Higham (2019) Supplementary Data 1, not in this paper's own tables: DeCasien describes them there as unpublished data the authors provided ("Sherwood et al.64 and Barks et al.65 provided neocortex, hippocampus, striatum, thalamus, cerebellum, amygdala and insula..."). So the VALUES ARE PUBLISHED - the item is keyed to the measuring paper's DOI, and the item number records the route. Renamed 2026-08-19 from 'unpublishedviaDeCasien', which wrongly implied the data itself is unpublished. Built and term-mapped; not yet in any volumes_compiled item list.</t>
+        </is>
+      </c>
+      <c r="AK19" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="AL19" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
       </c>
     </row>
     <row r="20" ht="16.5" customHeight="1">
@@ -10357,12 +10374,12 @@
       </c>
       <c r="AB59" t="inlineStr">
         <is>
-          <t>Data role = SECONDARY. Every macroanatomical column is re-used data: left V1 / left LGN / neocortex / brain mass = deSousa_etal_2010_Table1 (the same 9 specimens; audited 31 match, 1 mismatch, 4 one-sided within print precision); optic nerve cross-sectional area + eye half surface area = Stephan &amp; Frahm 1981 species means (footnote f); human neocortex = MacLeod unpublished combined-sex mean n = 8 (footnote b); ptd brain+body mass = Herndon et al. 1999 (footnote d); Homo body mass = Zilles 1972 (a); Pan paniscus body mass = Jungers &amp; Susman 1984 (c); EQ = derived (Martin 1981 / Ruff et al. 1997). The paper's own primary measurements (GLI values, relative laminar widths) are published only in Figures 5-7 and are not tabulated, and Tables 2-4 are derived statistics, so nothing here is ingested into a merge. Why the item is still worth having: it prints left V1 and left LGN in whole mm3 where 2010 Table 1 prints 1-d.p. cm3, and it confirms Macaca fascicularis ma22 left LGN = 46 mm3, which 2010 printed as 0 and the project had reconstructed as 0.046 cm3 from Supp. Table 2. All nine specimens resolve to the collection catalog (CAT-070, 080, 082, 095, 111, 131, 133, 134, 150) with printed sex and age matching. See deSousa_etal_2009_Table1.ReadMe.md.</t>
+          <t>Data role = SECONDARY. Every macroanatomical column is re-used data. The NEOCORTEX column is Carol MacLeod's own unpublished measurement (MacLeod_data.xls Table II, emailed 2002-09-15; held in the private repo as ____Unpublished__MacLeod_neocortex/ under her conditions of use - do not publish the raw neocortex values, and label specimens in the published JHE format). Its human value of 974 cm3 is the mean of her 8 humans (973.9987), which is footnote b. left V1 / left LGN / brain mass = deSousa_etal_2010_Table1, the same 9 specimens (audited 31 match, 1 mismatch, 4 one-sided within print precision). optic nerve cross-sectional area + eye half surface area = Stephan &amp; Frahm 1981 species means (footnote f). ptd brain+body mass = Herndon et al. 1999 (d); Homo body mass = Zilles 1972 (a); Pan paniscus body mass = Jungers &amp; Susman 1984 (c); EQ = derived (Martin 1981 / Ruff et al. 1997). The paper's own primary measurements (GLI values, relative laminar widths) are published only in Figures 5-7 and are not tabulated, and Tables 2-4 are derived statistics, so nothing here is ingested into a merge. Why the item is still worth having: it prints left V1 and left LGN in whole mm3 where 2010 Table 1 prints 1-d.p. cm3, and it confirms Macaca fascicularis ma22 left LGN = 46 mm3, which 2010 printed as 0 and the project had reconstructed as 0.046 cm3 from Supp. Table 2. All nine specimens resolve to the collection catalog (CAT-070, 080, 082, 095, 111, 131, 133, 134, 150) with printed sex and age matching. See deSousa_etal_2009_Table1.ReadMe.md.</t>
         </is>
       </c>
       <c r="AC59" t="inlineStr">
         <is>
-          <t>value-provenance: neocortex for ppz (Zahlia) printed as 279 cm3 is the value deSousa_etal_2010_Table1 gives for a DIFFERENT bonobo (YN86-137); Zahlia's own neocortex is 214.4 cm3. Kept as printed in the snapshot and the data, flagged, and not merged (plausible value belonging to a real sibling specimen, so it is not corrected by guesswork).  ||  laterality: left V1 + left LGN are LEFT hemisphere printed UNDOUBLED - registered in __merging_volumes/laterality_known.csv as doubling = none, required_suffix = _left.  ||  rounding vs deSousa_etal_2010_Table1: brain mass 58 g vs 57.6 g (mf2) and 360 g vs 359.5 g (ptb); neocortex 254 vs 254.3, 269 vs 268.5, 263 vs 262.8, 198 vs 198.3 cm3 - print rounding, not disagreement.  ||  derived-not-transcribed: Tables 2-4 (RMA regressions, Euclidean distances, PCA loadings) deliberately not built.</t>
+          <t>value-provenance: neocortex for ppz (Zahlia) printed as 279 cm3 is PAN PANISCUS H1 = YN86-137 (278.968) in Carol MacLeod's MacLeod_data.xls Table II; Zahlia is H2 (214.405). MECHANISM KNOWN: that sheet labels specimens anonymously (H1, H2, ...) with no archive numbers, and the 2009 table took the wrong H-row for the bonobo - the crosswalk resolving her H-numbers to named specimens is ____Unpublished__MacLeod_neocortex/MacLeod_specimen_crosswalk.csv in the private repo. Kept as printed in the snapshot and the data, flagged, not merged (a real measurement of a real specimen, printed against the wrong animal - not corrected by guesswork).  ||  laterality: left V1 + left LGN are LEFT hemisphere printed UNDOUBLED - registered in __merging_volumes/laterality_known.csv as doubling = none, required_suffix = _left.  ||  rounding vs deSousa_etal_2010_Table1: brain mass 58 g vs 57.6 g (mf2) and 360 g vs 359.5 g (ptb); neocortex 254 vs 254.3, 269 vs 268.5, 263 vs 262.8, 198 vs 198.3 cm3 - print rounding, not disagreement.  ||  derived-not-transcribed: Tables 2-4 (RMA regressions, Euclidean distances, PCA loadings) deliberately not built.</t>
         </is>
       </c>
       <c r="AF59" s="3" t="inlineStr">
@@ -22193,8 +22210,10 @@
         <v>877</v>
       </c>
       <c r="B225" s="3"/>
-      <c r="D225" s="3" t="s">
-        <v>102</v>
+      <c r="D225" s="3" t="inlineStr">
+        <is>
+          <t>viaDeCasien2019</t>
+        </is>
       </c>
       <c r="E225" s="2" t="str">
         <f t="shared" si="32"/>
@@ -22222,11 +22241,11 @@
       </c>
       <c r="K225" s="2" t="str">
         <f t="shared" si="38"/>
-        <v>Sherwood_etal_2004_unpublishedviaDeCasien</v>
+        <v>Sherwood_etal_2004_viaDeCasien2019</v>
       </c>
       <c r="L225" s="2" t="str">
         <f t="shared" si="39"/>
-        <v>10.1002%2Fajp.20048_unpublishedviaDeCasien</v>
+        <v>10.1002%2Fajp.20048_viaDeCasien2019</v>
       </c>
       <c r="M225" s="2" t="str">
         <f t="array" ref="M225">IFERROR(INDEX(AUTO_Public_TSV_FileList!$A$1:$A$1000,MATCH(TRUE(),EXACT(L225,IFERROR(_xlfn.TEXTBEFORE(AUTO_Public_TSV_FileList!$A$1:$A$1000,".tsv"),"")),0)),"notfound")</f>
@@ -22241,14 +22260,26 @@
       <c r="Z225" s="3" t="s">
         <v>881</v>
       </c>
+      <c r="AB225" t="inlineStr">
+        <is>
+          <t>Regional volumes measured by the Sherwood / Barks teams and published in DeCasien &amp; Higham (2019) Supplementary Data 1, not in this paper's own tables: DeCasien describes them there as unpublished data the authors provided ("Sherwood et al.64 and Barks et al.65 provided neocortex, hippocampus, striatum, thalamus, cerebellum, amygdala and insula..."). So the VALUES ARE PUBLISHED - the item is keyed to the measuring paper's DOI, and the item number records the route. Renamed 2026-08-19 from 'unpublishedviaDeCasien', which wrongly implied the data itself is unpublished. Built and term-mapped; not yet in any volumes_compiled item list.</t>
+        </is>
+      </c>
       <c r="AF225" s="3" t="s">
         <v>761</v>
       </c>
       <c r="AG225" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="AK225" s="3" t="s">
-        <v>62</v>
+      <c r="AK225" s="3" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="AL225" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
       </c>
     </row>
     <row r="226" ht="15" customHeight="1">

</xml_diff>

<commit_message>
Refresh Shiny app data 2026-09-03 08:13
</commit_message>
<xml_diff>
--- a/__ReadMe.xlsx
+++ b/__ReadMe.xlsx
@@ -4565,7 +4565,7 @@
     <t>MamPhy v1 DNA-only maximum clade credibility tree</t>
   </si>
   <si>
-    <t>Van Essen, D. C., Drury, H. A., &amp; New Collective, A. (1997). Structural and functional analyses of human cerebral cortex using a surface-based atlas. J Neurosci, 17(18), 7079-7102. https://doi.org/10.1523/JNEUROSCI.17-18-07079.1997</t>
+    <t xml:space="preserve">Van Essen, D. C., &amp; Drury, H. A. (1997). Structural and functional analyses of human cerebral cortex using a surface-based atlas. J Neurosci, 17(18), 7079-7102. https://doi.org/10.1523/JNEUROSCI.17-18-07079.1997</t>
   </si>
   <si>
     <t>Table 1. Surface area measurements of cortical lobes</t>
@@ -33605,7 +33605,7 @@
       </c>
       <c r="F357" s="12" t="str">
         <f t="shared" si="145"/>
-        <v>VanEssen_etal_1997</v>
+        <v>VanEssen_Drury_1997</v>
       </c>
       <c r="G357" s="12" t="str">
         <f t="shared" si="146"/>
@@ -33618,7 +33618,7 @@
 _xlpm.commasBeforeAmp,IF(_xlpm.hasAmp,LEN(_xlfn.TEXTBEFORE(_xlpm.authors,"&amp;"))-LEN(SUBSTITUTE(_xlfn.TEXTBEFORE(_xlpm.authors,"&amp;"),",","")),0),
 IF(NOT(_xlpm.hasAmp),"",IF(_xlpm.commasBeforeAmp&gt;2,"etal",TRIM(_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(_xlpm.authors,"&amp; "),","))))
 )</f>
-        <v>etal</v>
+        <v>Drury</v>
       </c>
       <c r="I357" s="12" t="str">
         <f t="shared" si="147"/>
@@ -33641,7 +33641,7 @@
       </c>
       <c r="K357" s="12" t="str">
         <f t="shared" si="148"/>
-        <v>VanEssen_etal_1997_Table1</v>
+        <v>VanEssen_Drury_1997_Table1</v>
       </c>
       <c r="L357" s="12" t="str">
         <f t="shared" si="149"/>

</xml_diff>